<commit_message>
Add Sep 23 Cornerstone and Heritage stat sheets.
</commit_message>
<xml_diff>
--- a/volleyball_stats.xlsx
+++ b/volleyball_stats.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="Player stats" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,10 +14,10 @@
     <sheet name="Definitions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Player stats'!$A$1:$X$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rotation stats'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Serving by set'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Matches'!$A$1:$D$1</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Player stats'!$A$1:$X$1</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Rotation stats'!$A$1:$P$1</definedName>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Serving by set'!$A$1:$K$1</definedName>
+    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Matches'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,9 +26,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt formatCode="YYYY-MM-DD" numFmtId="164"/>
+    <numFmt formatCode="0.000" numFmtId="165"/>
+    <numFmt formatCode="yyyy-mm-dd h:mm:ss" numFmtId="166"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -74,32 +74,32 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="14">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -460,36 +460,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X100"/>
+  <dimension ref="A1:X122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="36" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="17" customWidth="1" min="23" max="23"/>
-    <col width="28" customWidth="1" min="24" max="24"/>
+    <col customWidth="1" max="1" min="1" width="12"/>
+    <col customWidth="1" max="2" min="2" width="12"/>
+    <col customWidth="1" max="3" min="3" width="12"/>
+    <col customWidth="1" max="4" min="4" width="12"/>
+    <col customWidth="1" max="5" min="5" width="12"/>
+    <col customWidth="1" max="6" min="6" width="17"/>
+    <col customWidth="1" max="7" min="7" width="12"/>
+    <col customWidth="1" max="8" min="8" width="13"/>
+    <col customWidth="1" max="9" min="9" width="17"/>
+    <col customWidth="1" max="10" min="10" width="28"/>
+    <col customWidth="1" max="11" min="11" width="16"/>
+    <col customWidth="1" max="12" min="12" width="12"/>
+    <col customWidth="1" max="13" min="13" width="14"/>
+    <col customWidth="1" max="14" min="14" width="14"/>
+    <col customWidth="1" max="15" min="15" width="36"/>
+    <col customWidth="1" max="16" min="16" width="17"/>
+    <col customWidth="1" max="17" min="17" width="14"/>
+    <col customWidth="1" max="18" min="18" width="15"/>
+    <col customWidth="1" max="19" min="19" width="24"/>
+    <col customWidth="1" max="20" min="20" width="22"/>
+    <col customWidth="1" max="21" min="21" width="36"/>
+    <col customWidth="1" max="22" min="22" width="19"/>
+    <col customWidth="1" max="23" min="23" width="17"/>
+    <col customWidth="1" max="24" min="24" width="28"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -5950,9 +5950,1098 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Tea</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>6</v>
+      </c>
+      <c r="F101" t="n">
+        <v>11</v>
+      </c>
+      <c r="G101" t="n">
+        <v>4</v>
+      </c>
+      <c r="H101" t="n">
+        <v>1</v>
+      </c>
+      <c r="I101" s="12" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="J101" s="12" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="K101" t="n">
+        <v>19</v>
+      </c>
+      <c r="L101" t="n">
+        <v>7</v>
+      </c>
+      <c r="M101" t="n">
+        <v>3</v>
+      </c>
+      <c r="N101" s="4" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>5 3 5 2 5 0 0 5 3 2 3 3 3 0 5 5 3 5 2</t>
+        </is>
+      </c>
+      <c r="P101" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>1</v>
+      </c>
+      <c r="R101" t="n">
+        <v>1</v>
+      </c>
+      <c r="S101" t="n">
+        <v>20</v>
+      </c>
+      <c r="T101" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>0 3 0 1 0 0 0 2 0 3 2 0 3 3 3 1 3 3 3 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Agnes</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" t="n">
+        <v>4</v>
+      </c>
+      <c r="H102" t="n">
+        <v>2</v>
+      </c>
+      <c r="I102" s="12" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="J102" s="12" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="K102" t="n">
+        <v>4</v>
+      </c>
+      <c r="M102" t="n">
+        <v>3</v>
+      </c>
+      <c r="N102" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>0 0 3 0</t>
+        </is>
+      </c>
+      <c r="Q102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Shiloh</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>6</v>
+      </c>
+      <c r="F103" t="n">
+        <v>8</v>
+      </c>
+      <c r="G103" t="n">
+        <v>5</v>
+      </c>
+      <c r="H103" t="n">
+        <v>2</v>
+      </c>
+      <c r="I103" s="12" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="J103" s="12" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="K103" t="n">
+        <v>20</v>
+      </c>
+      <c r="L103" t="n">
+        <v>4</v>
+      </c>
+      <c r="M103" t="n">
+        <v>2</v>
+      </c>
+      <c r="N103" s="4" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="P103" t="n">
+        <v>1</v>
+      </c>
+      <c r="S103" t="n">
+        <v>17</v>
+      </c>
+      <c r="T103" s="4" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>0 2 2 2 2 1 3 1 2 1 3 2 0 2 3 0 1</t>
+        </is>
+      </c>
+      <c r="V103" t="n">
+        <v>6</v>
+      </c>
+      <c r="W103" s="4" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>2 3 1 2 3 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Bridget</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>2</v>
+      </c>
+      <c r="F104" t="n">
+        <v>2</v>
+      </c>
+      <c r="I104" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" t="n">
+        <v>5</v>
+      </c>
+      <c r="L104" t="n">
+        <v>1</v>
+      </c>
+      <c r="M104" t="n">
+        <v>1</v>
+      </c>
+      <c r="N104" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>3 3 5 0 2</t>
+        </is>
+      </c>
+      <c r="P104" t="n">
+        <v>1</v>
+      </c>
+      <c r="S104" t="n">
+        <v>5</v>
+      </c>
+      <c r="T104" s="4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>1 0 3 1 3</t>
+        </is>
+      </c>
+      <c r="V104" t="n">
+        <v>3</v>
+      </c>
+      <c r="W104" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>2 2 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Corena</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>2</v>
+      </c>
+      <c r="E105" t="n">
+        <v>9</v>
+      </c>
+      <c r="F105" t="n">
+        <v>3</v>
+      </c>
+      <c r="I105" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="n">
+        <v>5</v>
+      </c>
+      <c r="V105" t="n">
+        <v>1</v>
+      </c>
+      <c r="W105" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>10</v>
+      </c>
+      <c r="K106" t="n">
+        <v>4</v>
+      </c>
+      <c r="M106" t="n">
+        <v>1</v>
+      </c>
+      <c r="N106" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="S106" t="n">
+        <v>20</v>
+      </c>
+      <c r="T106" s="4" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>1 0 2 0 1 0 2 3 2 3 2 3 3 1 0 0 0 0 0 0</t>
+        </is>
+      </c>
+      <c r="V106" t="n">
+        <v>4</v>
+      </c>
+      <c r="W106" s="4" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Addy</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
+      </c>
+      <c r="I107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" t="n">
+        <v>20</v>
+      </c>
+      <c r="L107" t="n">
+        <v>7</v>
+      </c>
+      <c r="M107" t="n">
+        <v>4</v>
+      </c>
+      <c r="N107" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>5 5 2 5 3 3 2 3 2 5 2 0 5 0 5 0 3 5 1 0</t>
+        </is>
+      </c>
+      <c r="R107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Nataly</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>3</v>
+      </c>
+      <c r="E108" t="n">
+        <v>4</v>
+      </c>
+      <c r="F108" t="n">
+        <v>2</v>
+      </c>
+      <c r="I108" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K108" t="n">
+        <v>12</v>
+      </c>
+      <c r="L108" t="n">
+        <v>6</v>
+      </c>
+      <c r="M108" t="n">
+        <v>2</v>
+      </c>
+      <c r="N108" s="4" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>5 3 5 0 2 3 5 0 5 5 3 5</t>
+        </is>
+      </c>
+      <c r="P108" t="n">
+        <v>4</v>
+      </c>
+      <c r="V108" t="n">
+        <v>4</v>
+      </c>
+      <c r="W108" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>1 1 2 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" t="n">
+        <v>11</v>
+      </c>
+      <c r="G109" t="n">
+        <v>4</v>
+      </c>
+      <c r="H109" t="n">
+        <v>1</v>
+      </c>
+      <c r="I109" s="12" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="J109" s="12" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="P109" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Gaby</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>1</v>
+      </c>
+      <c r="H110" t="n">
+        <v>1</v>
+      </c>
+      <c r="I110" s="12" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J110" s="12" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S110" t="n">
+        <v>2</v>
+      </c>
+      <c r="T110" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>0 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Annabelle</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>2</v>
+      </c>
+      <c r="F111" t="n">
+        <v>5</v>
+      </c>
+      <c r="G111" t="n">
+        <v>2</v>
+      </c>
+      <c r="I111" s="12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J111" s="12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K111" t="n">
+        <v>6</v>
+      </c>
+      <c r="L111" t="n">
+        <v>2</v>
+      </c>
+      <c r="M111" t="n">
+        <v>4</v>
+      </c>
+      <c r="N111" s="4" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>0 0 5 5 0 0</t>
+        </is>
+      </c>
+      <c r="P111" t="n">
+        <v>2</v>
+      </c>
+      <c r="S111" t="n">
+        <v>7</v>
+      </c>
+      <c r="T111" s="4" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>0 0 0 2 3 0 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Shiloh</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>3</v>
+      </c>
+      <c r="F112" t="n">
+        <v>12</v>
+      </c>
+      <c r="G112" t="n">
+        <v>3</v>
+      </c>
+      <c r="H112" t="n">
+        <v>3</v>
+      </c>
+      <c r="I112" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J112" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K112" t="n">
+        <v>15</v>
+      </c>
+      <c r="L112" t="n">
+        <v>8</v>
+      </c>
+      <c r="N112" s="4" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>5 5 3 5 5 5 2 5 5 5 1 3 3 3 3</t>
+        </is>
+      </c>
+      <c r="P112" t="n">
+        <v>2</v>
+      </c>
+      <c r="S112" t="n">
+        <v>15</v>
+      </c>
+      <c r="T112" s="4" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>2 0 2 3 2 1 3 2 1 0 0 2 1 2 2</t>
+        </is>
+      </c>
+      <c r="V112" t="n">
+        <v>5</v>
+      </c>
+      <c r="W112" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>3 1 2 2 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>2</v>
+      </c>
+      <c r="K113" t="n">
+        <v>8</v>
+      </c>
+      <c r="L113" t="n">
+        <v>1</v>
+      </c>
+      <c r="M113" t="n">
+        <v>2</v>
+      </c>
+      <c r="N113" s="4" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>3 5 1 3 0 1 2 0</t>
+        </is>
+      </c>
+      <c r="S113" t="n">
+        <v>8</v>
+      </c>
+      <c r="T113" s="4" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>0 2 3 3 1 0 2 2</t>
+        </is>
+      </c>
+      <c r="V113" t="n">
+        <v>2</v>
+      </c>
+      <c r="W113" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>2 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Annabelle</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>5</v>
+      </c>
+      <c r="E114" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" t="n">
+        <v>7</v>
+      </c>
+      <c r="G114" t="n">
+        <v>4</v>
+      </c>
+      <c r="H114" t="n">
+        <v>1</v>
+      </c>
+      <c r="I114" s="12" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="J114" s="12" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="K114" t="n">
+        <v>9</v>
+      </c>
+      <c r="L114" t="n">
+        <v>1</v>
+      </c>
+      <c r="M114" t="n">
+        <v>2</v>
+      </c>
+      <c r="N114" s="4" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>2 3 0 5 2 2 0 2 3</t>
+        </is>
+      </c>
+      <c r="S114" t="n">
+        <v>2</v>
+      </c>
+      <c r="T114" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>2 1</t>
+        </is>
+      </c>
+      <c r="V114" t="n">
+        <v>3</v>
+      </c>
+      <c r="W114" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>2 2 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>10</v>
+      </c>
+      <c r="G115" t="n">
+        <v>3</v>
+      </c>
+      <c r="I115" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J115" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Nataly</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>4</v>
+      </c>
+      <c r="E116" t="n">
+        <v>7</v>
+      </c>
+      <c r="F116" t="n">
+        <v>4</v>
+      </c>
+      <c r="G116" t="n">
+        <v>2</v>
+      </c>
+      <c r="I116" s="12" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="J116" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K116" t="n">
+        <v>10</v>
+      </c>
+      <c r="L116" t="n">
+        <v>3</v>
+      </c>
+      <c r="M116" t="n">
+        <v>1</v>
+      </c>
+      <c r="N116" s="4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>2 5 5 0 1 1 1 5 3 3</t>
+        </is>
+      </c>
+      <c r="P116" t="n">
+        <v>3</v>
+      </c>
+      <c r="V116" t="n">
+        <v>1</v>
+      </c>
+      <c r="W116" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="X116" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Tea</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>2</v>
+      </c>
+      <c r="E117" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" t="n">
+        <v>7</v>
+      </c>
+      <c r="G117" t="n">
+        <v>2</v>
+      </c>
+      <c r="I117" s="12" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="J117" s="12" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="K117" t="n">
+        <v>17</v>
+      </c>
+      <c r="L117" t="n">
+        <v>9</v>
+      </c>
+      <c r="M117" t="n">
+        <v>2</v>
+      </c>
+      <c r="N117" s="4" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>3 5 3 3 5 5 3 5 5 2 5 5 2 5 0 5 0</t>
+        </is>
+      </c>
+      <c r="P117" t="n">
+        <v>1</v>
+      </c>
+      <c r="S117" t="n">
+        <v>13</v>
+      </c>
+      <c r="T117" s="4" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>3 1 2 1 2 2 3 1 3 3 1 3 3</t>
+        </is>
+      </c>
+      <c r="V117" t="n">
+        <v>1</v>
+      </c>
+      <c r="W117" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Addy</t>
+        </is>
+      </c>
+      <c r="K118" t="n">
+        <v>11</v>
+      </c>
+      <c r="L118" t="n">
+        <v>4</v>
+      </c>
+      <c r="M118" t="n">
+        <v>3</v>
+      </c>
+      <c r="N118" s="4" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>0 0 5 3 1 5 5 2 5 3 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Agnes</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>4</v>
+      </c>
+      <c r="G119" t="n">
+        <v>3</v>
+      </c>
+      <c r="I119" s="12" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J119" s="12" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Bridget</t>
+        </is>
+      </c>
+      <c r="S120" t="n">
+        <v>2</v>
+      </c>
+      <c r="T120" s="4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>2 3</t>
+        </is>
+      </c>
+      <c r="V120" t="n">
+        <v>3</v>
+      </c>
+      <c r="W120" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>0 3 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Elena</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>1</v>
+      </c>
+      <c r="I121" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Corena</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:X1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -5965,25 +7054,25 @@
   <dimension ref="A1:P43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col customWidth="1" max="1" min="1" width="12"/>
+    <col customWidth="1" max="2" min="2" width="12"/>
+    <col customWidth="1" max="3" min="3" width="12"/>
+    <col customWidth="1" max="4" min="4" width="12"/>
+    <col customWidth="1" max="5" min="5" width="17"/>
+    <col customWidth="1" max="6" min="6" width="12"/>
+    <col customWidth="1" max="7" min="7" width="13"/>
+    <col customWidth="1" max="8" min="8" width="17"/>
+    <col customWidth="1" max="9" min="9" width="17"/>
+    <col customWidth="1" max="10" min="10" width="24"/>
+    <col customWidth="1" max="11" min="11" width="23"/>
+    <col customWidth="1" max="12" min="12" width="12"/>
+    <col customWidth="1" max="13" min="13" width="14"/>
+    <col customWidth="1" max="14" min="14" width="15"/>
+    <col customWidth="1" max="15" min="15" width="16"/>
+    <col customWidth="1" max="16" min="16" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -8173,7 +9262,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -8183,23 +9272,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col customWidth="1" max="1" min="1" width="12"/>
+    <col customWidth="1" max="2" min="2" width="12"/>
+    <col customWidth="1" max="3" min="3" width="12"/>
+    <col customWidth="1" max="4" min="4" width="12"/>
+    <col customWidth="1" max="5" min="5" width="19"/>
+    <col customWidth="1" max="6" min="6" width="12"/>
+    <col customWidth="1" max="7" min="7" width="20"/>
+    <col customWidth="1" max="8" min="8" width="13"/>
+    <col customWidth="1" max="9" min="9" width="21"/>
+    <col customWidth="1" max="10" min="10" width="14"/>
+    <col customWidth="1" max="11" min="11" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -9504,9 +10593,287 @@
         <v>0.11</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" t="n">
+        <v>5</v>
+      </c>
+      <c r="H46" t="n">
+        <v>7</v>
+      </c>
+      <c r="I46" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" t="n">
+        <v>6</v>
+      </c>
+      <c r="H47" t="n">
+        <v>9</v>
+      </c>
+      <c r="I47" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" t="n">
+        <v>4</v>
+      </c>
+      <c r="H48" t="n">
+        <v>7</v>
+      </c>
+      <c r="I48" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="n">
+        <v>9</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>5</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" t="n">
+        <v>3</v>
+      </c>
+      <c r="H50" t="n">
+        <v>8</v>
+      </c>
+      <c r="I50" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F51" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H51" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="J51" s="7" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="K51" s="7" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>11</v>
+      </c>
+      <c r="E52" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" t="n">
+        <v>5</v>
+      </c>
+      <c r="I52" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="n">
+        <v>9</v>
+      </c>
+      <c r="E53" t="n">
+        <v>2</v>
+      </c>
+      <c r="H53" t="n">
+        <v>2</v>
+      </c>
+      <c r="I53" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+      <c r="H54" t="n">
+        <v>5</v>
+      </c>
+      <c r="I54" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H55" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I55" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J55" s="7" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K55" s="7" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -9516,16 +10883,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col customWidth="1" max="1" min="1" width="12"/>
+    <col customWidth="1" max="2" min="2" width="12"/>
+    <col customWidth="1" max="3" min="3" width="22"/>
+    <col customWidth="1" max="4" min="4" width="28"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -9669,9 +11036,35 @@
         <v>-0.014</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cornerstone</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>0.167</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>0.289</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -9684,8 +11077,8 @@
   <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col customWidth="1" max="1" min="1" width="36"/>
+    <col customWidth="1" max="2" min="2" width="110"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9700,7 +11093,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Blank cells</t>
@@ -9712,7 +11105,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Digs</t>
@@ -9724,7 +11117,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Assists</t>
@@ -9736,7 +11129,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Attack attempts, Kills, Kill errors</t>
@@ -9748,7 +11141,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Kill efficiency</t>
@@ -9760,7 +11153,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Kill efficiency (calculated)</t>
@@ -9772,7 +11165,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Serve attempts, Aces, Serve errors</t>
@@ -9784,7 +11177,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Serve rating</t>
@@ -9796,7 +11189,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Serving scores</t>
@@ -9808,7 +11201,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Unforced errors</t>
@@ -9820,7 +11213,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Stuff blocks</t>
@@ -9832,7 +11225,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Block touches</t>
@@ -9844,7 +11237,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Serve receive rating</t>
@@ -9856,7 +11249,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Serve receive grades</t>
@@ -9868,7 +11261,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Freeball attempts / rating / grades</t>
@@ -9880,7 +11273,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Rotation</t>
@@ -9892,7 +11285,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Points scored / against / net</t>
@@ -9904,7 +11297,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Serving by set</t>
@@ -9916,7 +11309,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Team kill efficiency</t>
@@ -9928,7 +11321,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
+    <row customHeight="1" ht="32" r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Note</t>
@@ -9941,6 +11334,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update stats from Google Sheet
</commit_message>
<xml_diff>
--- a/volleyball_stats.xlsx
+++ b/volleyball_stats.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Player stats" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,10 +14,10 @@
     <sheet name="Definitions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Player stats'!$A$1:$X$1</definedName>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Rotation stats'!$A$1:$P$1</definedName>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Serving by set'!$A$1:$K$1</definedName>
-    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Matches'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Player stats'!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rotation stats'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Serving by set'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Matches'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,9 +26,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt formatCode="YYYY-MM-DD" numFmtId="164"/>
-    <numFmt formatCode="0.000" numFmtId="165"/>
-    <numFmt formatCode="yyyy-mm-dd h:mm:ss" numFmtId="166"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -74,33 +74,33 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="15">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="165" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="166" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -461,36 +461,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X222"/>
+  <dimension ref="A1:X224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="12"/>
-    <col customWidth="1" max="2" min="2" width="12"/>
-    <col customWidth="1" max="3" min="3" width="12"/>
-    <col customWidth="1" max="4" min="4" width="12"/>
-    <col customWidth="1" max="5" min="5" width="12"/>
-    <col customWidth="1" max="6" min="6" width="17"/>
-    <col customWidth="1" max="7" min="7" width="12"/>
-    <col customWidth="1" max="8" min="8" width="13"/>
-    <col customWidth="1" max="9" min="9" width="17"/>
-    <col customWidth="1" max="10" min="10" width="28"/>
-    <col customWidth="1" max="11" min="11" width="16"/>
-    <col customWidth="1" max="12" min="12" width="12"/>
-    <col customWidth="1" max="13" min="13" width="14"/>
-    <col customWidth="1" max="14" min="14" width="14"/>
-    <col customWidth="1" max="15" min="15" width="36"/>
-    <col customWidth="1" max="16" min="16" width="17"/>
-    <col customWidth="1" max="17" min="17" width="14"/>
-    <col customWidth="1" max="18" min="18" width="15"/>
-    <col customWidth="1" max="19" min="19" width="24"/>
-    <col customWidth="1" max="20" min="20" width="22"/>
-    <col customWidth="1" max="21" min="21" width="36"/>
-    <col customWidth="1" max="22" min="22" width="19"/>
-    <col customWidth="1" max="23" min="23" width="17"/>
-    <col customWidth="1" max="24" min="24" width="28"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="36" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="28" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="32" r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -11417,6 +11417,9 @@
       <c r="S205" t="n">
         <v>22</v>
       </c>
+      <c r="T205" t="n">
+        <v>1.45</v>
+      </c>
       <c r="U205" t="inlineStr">
         <is>
           <t>2 3 0 2 1 2 3 2 3 1 3 2 2 0 2 0 1 1 0 0 1 1</t>
@@ -11424,6 +11427,9 @@
       </c>
       <c r="V205" t="n">
         <v>4</v>
+      </c>
+      <c r="W205" t="n">
+        <v>2.5</v>
       </c>
       <c r="X205" t="inlineStr">
         <is>
@@ -11469,6 +11475,9 @@
       <c r="M206" t="n">
         <v>3</v>
       </c>
+      <c r="N206" t="n">
+        <v>2.82</v>
+      </c>
       <c r="O206" t="inlineStr">
         <is>
           <t>5 5 5 3 5 3 0 2 0 3 0</t>
@@ -11516,6 +11525,9 @@
       <c r="K207" t="n">
         <v>1</v>
       </c>
+      <c r="N207" t="n">
+        <v>3</v>
+      </c>
       <c r="O207" t="inlineStr">
         <is>
           <t>3</t>
@@ -11525,6 +11537,9 @@
         <v>4</v>
       </c>
       <c r="V207" t="n">
+        <v>1</v>
+      </c>
+      <c r="W207" t="n">
         <v>1</v>
       </c>
       <c r="X207" t="inlineStr">
@@ -11577,6 +11592,9 @@
       <c r="M208" t="n">
         <v>2</v>
       </c>
+      <c r="N208" t="n">
+        <v>2.63</v>
+      </c>
       <c r="O208" t="inlineStr">
         <is>
           <t>2 0 5 1 3 5 5 3 2 3 3 3 1 5 1 5 0 1 2</t>
@@ -11588,6 +11606,9 @@
       <c r="S208" t="n">
         <v>17</v>
       </c>
+      <c r="T208" t="n">
+        <v>1.71</v>
+      </c>
       <c r="U208" t="inlineStr">
         <is>
           <t>1 1 3 2 3 3 2 1 2 2 1 0 1 2 3 0 2</t>
@@ -11595,6 +11616,9 @@
       </c>
       <c r="V208" t="n">
         <v>4</v>
+      </c>
+      <c r="W208" t="n">
+        <v>2.5</v>
       </c>
       <c r="X208" t="inlineStr">
         <is>
@@ -11637,6 +11661,9 @@
       <c r="L209" t="n">
         <v>4</v>
       </c>
+      <c r="N209" t="n">
+        <v>2.65</v>
+      </c>
       <c r="O209" t="inlineStr">
         <is>
           <t>2 5 2 1 2 1 5 3 2 1 2 3 1 5 2 3 3 3 5 2</t>
@@ -11648,6 +11675,9 @@
       <c r="S209" t="n">
         <v>20</v>
       </c>
+      <c r="T209" t="n">
+        <v>1</v>
+      </c>
       <c r="U209" t="inlineStr">
         <is>
           <t>1 2 2 1 0 0 0 0 2 1 0 3 0 2 1 2 1 0 2 0</t>
@@ -11655,6 +11685,9 @@
       </c>
       <c r="V209" t="n">
         <v>1</v>
+      </c>
+      <c r="W209" t="n">
+        <v>2</v>
       </c>
       <c r="X209" t="inlineStr">
         <is>
@@ -11742,6 +11775,9 @@
       <c r="M211" t="n">
         <v>3</v>
       </c>
+      <c r="N211" t="n">
+        <v>2.75</v>
+      </c>
       <c r="O211" t="inlineStr">
         <is>
           <t>3 1 5 1 5 5 0 5 0 5 0 3</t>
@@ -11752,6 +11788,9 @@
       </c>
       <c r="S211" t="n">
         <v>5</v>
+      </c>
+      <c r="T211" t="n">
+        <v>0.6</v>
       </c>
       <c r="U211" t="inlineStr">
         <is>
@@ -11760,6 +11799,9 @@
       </c>
       <c r="V211" t="n">
         <v>6</v>
+      </c>
+      <c r="W211" t="n">
+        <v>1.83</v>
       </c>
       <c r="X211" t="inlineStr">
         <is>
@@ -11790,6 +11832,9 @@
       <c r="M212" t="n">
         <v>2</v>
       </c>
+      <c r="N212" t="n">
+        <v>2</v>
+      </c>
       <c r="O212" t="inlineStr">
         <is>
           <t>5 2 0 3 0</t>
@@ -11828,6 +11873,9 @@
       <c r="L213" t="n">
         <v>1</v>
       </c>
+      <c r="N213" t="n">
+        <v>3.67</v>
+      </c>
       <c r="O213" t="inlineStr">
         <is>
           <t>3 5 3</t>
@@ -11852,36 +11900,60 @@
         </is>
       </c>
       <c r="D214" t="n">
+        <v>10</v>
+      </c>
+      <c r="F214" t="n">
+        <v>1</v>
+      </c>
+      <c r="G214" t="n">
+        <v>1</v>
+      </c>
+      <c r="I214" t="n">
+        <v>1</v>
+      </c>
+      <c r="J214" t="n">
         <v>1</v>
       </c>
       <c r="K214" t="n">
-        <v>3</v>
+        <v>12</v>
+      </c>
+      <c r="L214" t="n">
+        <v>2</v>
       </c>
       <c r="M214" t="n">
         <v>2</v>
       </c>
+      <c r="N214" t="n">
+        <v>2.58</v>
+      </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>3 0 0</t>
+          <t>3 0 0 3 3 2 5 5 1 3 3 3</t>
         </is>
       </c>
       <c r="P214" t="n">
         <v>1</v>
       </c>
       <c r="S214" t="n">
-        <v>13</v>
+        <v>24</v>
+      </c>
+      <c r="T214" t="n">
+        <v>1.46</v>
       </c>
       <c r="U214" t="inlineStr">
         <is>
-          <t>1 2 3 0 1 1 0 0 1 2 3 1 2</t>
+          <t>1 2 3 0 1 1 0 0 1 2 3 1 2 0 2 2 1 1 3 3 1 1 3 1</t>
         </is>
       </c>
       <c r="V214" t="n">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="W214" t="n">
+        <v>2.58</v>
       </c>
       <c r="X214" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2 3 2 3 3 3 2 3 3 3 2 2</t>
         </is>
       </c>
     </row>
@@ -11900,48 +11972,66 @@
         </is>
       </c>
       <c r="D215" t="n">
+        <v>11</v>
+      </c>
+      <c r="E215" t="n">
+        <v>4</v>
+      </c>
+      <c r="F215" t="n">
+        <v>16</v>
+      </c>
+      <c r="G215" t="n">
+        <v>3</v>
+      </c>
+      <c r="H215" t="n">
+        <v>4</v>
+      </c>
+      <c r="I215" t="n">
+        <v>-0.063</v>
+      </c>
+      <c r="J215" t="n">
+        <v>-0.062</v>
+      </c>
+      <c r="K215" t="n">
+        <v>13</v>
+      </c>
+      <c r="L215" t="n">
+        <v>3</v>
+      </c>
+      <c r="M215" t="n">
+        <v>7</v>
+      </c>
+      <c r="N215" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>5 5 5 0 0 3 1 0 0 0 2 0 0</t>
+        </is>
+      </c>
+      <c r="P215" t="n">
+        <v>3</v>
+      </c>
+      <c r="S215" t="n">
         <v>6</v>
       </c>
-      <c r="F215" t="n">
-        <v>7</v>
-      </c>
-      <c r="G215" t="n">
-        <v>1</v>
-      </c>
-      <c r="H215" t="n">
-        <v>3</v>
-      </c>
-      <c r="J215" t="n">
-        <v>-0.286</v>
-      </c>
-      <c r="K215" t="n">
-        <v>7</v>
-      </c>
-      <c r="L215" t="n">
-        <v>3</v>
-      </c>
-      <c r="M215" t="n">
-        <v>2</v>
-      </c>
-      <c r="O215" t="inlineStr">
-        <is>
-          <t>5 5 5 0 0 3 1</t>
-        </is>
-      </c>
-      <c r="S215" t="n">
-        <v>2</v>
+      <c r="T215" t="n">
+        <v>1.17</v>
       </c>
       <c r="U215" t="inlineStr">
         <is>
-          <t>0 1</t>
+          <t>0 1 0 2 3 1</t>
         </is>
       </c>
       <c r="V215" t="n">
-        <v>3</v>
+        <v>11</v>
+      </c>
+      <c r="W215" t="n">
+        <v>2.36</v>
       </c>
       <c r="X215" t="inlineStr">
         <is>
-          <t>3 2 2</t>
+          <t>3 2 2 1 3 2 3 3 2 3 2</t>
         </is>
       </c>
     </row>
@@ -11959,35 +12049,53 @@
           <t>Nataly</t>
         </is>
       </c>
+      <c r="D216" t="n">
+        <v>6</v>
+      </c>
       <c r="E216" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F216" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="G216" t="n">
+        <v>1</v>
+      </c>
+      <c r="I216" t="n">
+        <v>0.5</v>
       </c>
       <c r="J216" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K216" t="n">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="L216" t="n">
+        <v>1</v>
       </c>
       <c r="M216" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="N216" t="n">
+        <v>2</v>
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>3 0</t>
+          <t>3 0 3 2 5 0 0 2 3 2</t>
         </is>
       </c>
       <c r="P216" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="V216" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="W216" t="n">
+        <v>2.5</v>
       </c>
       <c r="X216" t="inlineStr">
         <is>
-          <t>2 3 3</t>
+          <t>2 3 3 3 3 1</t>
         </is>
       </c>
     </row>
@@ -12006,54 +12114,66 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E217" t="n">
         <v>1</v>
       </c>
       <c r="F217" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="G217" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="H217" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="I217" t="n">
+        <v>0.326</v>
       </c>
       <c r="J217" t="n">
-        <v>0.333</v>
+        <v>0.326</v>
       </c>
       <c r="K217" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="L217" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M217" t="n">
         <v>1</v>
       </c>
+      <c r="N217" t="n">
+        <v>2.86</v>
+      </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2 5 3 3 3 3 3 2 2 5 2 0</t>
+          <t>2 5 3 3 3 3 3 2 2 5 2 0 3 2 3 5 1 2 3 5 3 3 3 3 3 3 3 2</t>
         </is>
       </c>
       <c r="P217" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S217" t="n">
-        <v>10</v>
+        <v>32</v>
+      </c>
+      <c r="T217" t="n">
+        <v>1.59</v>
       </c>
       <c r="U217" t="inlineStr">
         <is>
-          <t>2 2 2 3 0 2 2 0 2 2</t>
+          <t>2 2 2 3 0 2 2 0 2 2 2 1 2 3 3 0 1 3 1 0 1 3 1 2 1 2 2 2 0 1 2 1</t>
         </is>
       </c>
       <c r="V217" t="n">
-        <v>6</v>
+        <v>23</v>
+      </c>
+      <c r="W217" t="n">
+        <v>2.43</v>
       </c>
       <c r="X217" t="inlineStr">
         <is>
-          <t>3 3 3 3 2 2</t>
+          <t>3 3 3 3 2 2 2 3 2 3 2 2 3 3 2 3 1 3 2 3 2 2 2</t>
         </is>
       </c>
     </row>
@@ -12072,42 +12192,57 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F218" t="n">
+        <v>33</v>
+      </c>
+      <c r="G218" t="n">
         <v>11</v>
       </c>
-      <c r="G218" t="n">
-        <v>3</v>
+      <c r="H218" t="n">
+        <v>1</v>
+      </c>
+      <c r="I218" t="n">
+        <v>0.303</v>
       </c>
       <c r="J218" t="n">
-        <v>0.273</v>
+        <v>0.303</v>
       </c>
       <c r="K218" t="n">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="N218" t="n">
+        <v>2.33</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2 3 3</t>
+          <t>2 3 3 1 2 3 2 2 3 2 2 3 2 3 2</t>
         </is>
       </c>
       <c r="P218" t="n">
         <v>1</v>
       </c>
       <c r="S218" t="n">
-        <v>7</v>
+        <v>19</v>
+      </c>
+      <c r="T218" t="n">
+        <v>1.79</v>
       </c>
       <c r="U218" t="inlineStr">
         <is>
-          <t>3 2 3 0 3 2 2</t>
+          <t>3 2 3 0 3 2 2 2 3 2 3 2 1 0 1 0 2 1 2</t>
         </is>
       </c>
       <c r="V218" t="n">
-        <v>2</v>
+        <v>17</v>
+      </c>
+      <c r="W218" t="n">
+        <v>2.47</v>
       </c>
       <c r="X218" t="inlineStr">
         <is>
-          <t>3 3</t>
+          <t>3 3 2 3 2 3 3 3 3 1 0 3 3 3 2 2 3</t>
         </is>
       </c>
     </row>
@@ -12125,22 +12260,37 @@
           <t>Agnes</t>
         </is>
       </c>
+      <c r="D219" t="n">
+        <v>3</v>
+      </c>
+      <c r="E219" t="n">
+        <v>1</v>
+      </c>
       <c r="F219" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G219" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H219" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="I219" t="n">
+        <v>0.063</v>
       </c>
       <c r="J219" t="n">
-        <v>0.167</v>
+        <v>0.062</v>
+      </c>
+      <c r="P219" t="n">
+        <v>2</v>
       </c>
       <c r="R219" t="n">
         <v>1</v>
       </c>
       <c r="V219" t="n">
+        <v>1</v>
+      </c>
+      <c r="W219" t="n">
         <v>1</v>
       </c>
       <c r="X219" t="inlineStr">
@@ -12164,33 +12314,45 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F220" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H220" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I220" t="n">
+        <v>-0.5</v>
       </c>
       <c r="J220" t="n">
         <v>-0.5</v>
       </c>
       <c r="K220" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="L220" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M220" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="N220" t="n">
+        <v>2.76</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>5 5 3 0 0 5 5 1</t>
-        </is>
+          <t>5 5 3 0 0 5 5 1 3 5 3 2 3 0 2 5 0</t>
+        </is>
+      </c>
+      <c r="R220" t="n">
+        <v>1</v>
       </c>
       <c r="S220" t="n">
         <v>2</v>
+      </c>
+      <c r="T220" t="n">
+        <v>1</v>
       </c>
       <c r="U220" t="inlineStr">
         <is>
@@ -12216,22 +12378,25 @@
         <v>1</v>
       </c>
       <c r="F221" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G221" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H221" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I221" t="n">
+        <v>0.111</v>
       </c>
       <c r="J221" t="n">
-        <v>0</v>
+        <v>0.111</v>
       </c>
       <c r="P221" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R221" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="222">
@@ -12248,10 +12413,77 @@
           <t>Corena</t>
         </is>
       </c>
+      <c r="D222" t="n">
+        <v>1</v>
+      </c>
+      <c r="E222" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="14" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Whitefield</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Gaby</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>2</v>
+      </c>
+      <c r="V223" t="n">
+        <v>2</v>
+      </c>
+      <c r="W223" t="n">
+        <v>2</v>
+      </c>
+      <c r="X223" t="inlineStr">
+        <is>
+          <t>3 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="14" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Whitefield</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Bridget</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>1</v>
+      </c>
+      <c r="P224" t="n">
+        <v>1</v>
+      </c>
+      <c r="V224" t="n">
+        <v>1</v>
+      </c>
+      <c r="W224" t="n">
+        <v>2</v>
+      </c>
+      <c r="X224" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:X1"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -12264,25 +12496,25 @@
   <dimension ref="A1:P85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="12"/>
-    <col customWidth="1" max="2" min="2" width="12"/>
-    <col customWidth="1" max="3" min="3" width="12"/>
-    <col customWidth="1" max="4" min="4" width="12"/>
-    <col customWidth="1" max="5" min="5" width="17"/>
-    <col customWidth="1" max="6" min="6" width="12"/>
-    <col customWidth="1" max="7" min="7" width="13"/>
-    <col customWidth="1" max="8" min="8" width="17"/>
-    <col customWidth="1" max="9" min="9" width="17"/>
-    <col customWidth="1" max="10" min="10" width="24"/>
-    <col customWidth="1" max="11" min="11" width="23"/>
-    <col customWidth="1" max="12" min="12" width="12"/>
-    <col customWidth="1" max="13" min="13" width="14"/>
-    <col customWidth="1" max="14" min="14" width="15"/>
-    <col customWidth="1" max="15" min="15" width="16"/>
-    <col customWidth="1" max="16" min="16" width="14"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="32" r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -16335,7 +16567,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -16348,20 +16580,20 @@
   <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="12"/>
-    <col customWidth="1" max="2" min="2" width="12"/>
-    <col customWidth="1" max="3" min="3" width="12"/>
-    <col customWidth="1" max="4" min="4" width="12"/>
-    <col customWidth="1" max="5" min="5" width="19"/>
-    <col customWidth="1" max="6" min="6" width="12"/>
-    <col customWidth="1" max="7" min="7" width="20"/>
-    <col customWidth="1" max="8" min="8" width="13"/>
-    <col customWidth="1" max="9" min="9" width="21"/>
-    <col customWidth="1" max="10" min="10" width="14"/>
-    <col customWidth="1" max="11" min="11" width="22"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="32" r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -19329,6 +19561,30 @@
           <t>Total</t>
         </is>
       </c>
+      <c r="D115" t="n">
+        <v>22</v>
+      </c>
+      <c r="E115" t="n">
+        <v>9</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H115" t="n">
+        <v>22</v>
+      </c>
+      <c r="I115" t="n">
+        <v>17</v>
+      </c>
+      <c r="J115" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="K115" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="n">
@@ -19374,10 +19630,10 @@
         <v>4</v>
       </c>
       <c r="H117" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I117" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118">
@@ -19392,6 +19648,18 @@
       <c r="C118" t="n">
         <v>3</v>
       </c>
+      <c r="D118" t="n">
+        <v>3</v>
+      </c>
+      <c r="E118" t="n">
+        <v>3</v>
+      </c>
+      <c r="H118" t="n">
+        <v>4</v>
+      </c>
+      <c r="I118" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="14" t="n">
@@ -19405,6 +19673,18 @@
       <c r="C119" t="n">
         <v>4</v>
       </c>
+      <c r="D119" t="n">
+        <v>2</v>
+      </c>
+      <c r="E119" t="n">
+        <v>2</v>
+      </c>
+      <c r="H119" t="n">
+        <v>1</v>
+      </c>
+      <c r="I119" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="n">
@@ -19418,6 +19698,18 @@
       <c r="C120" t="n">
         <v>5</v>
       </c>
+      <c r="D120" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" t="n">
+        <v>2</v>
+      </c>
+      <c r="H120" t="n">
+        <v>4</v>
+      </c>
+      <c r="I120" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="14" t="n">
@@ -19433,10 +19725,34 @@
           <t>Total</t>
         </is>
       </c>
+      <c r="D121" t="n">
+        <v>15</v>
+      </c>
+      <c r="E121" t="n">
+        <v>14</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H121" t="n">
+        <v>19</v>
+      </c>
+      <c r="I121" t="n">
+        <v>14</v>
+      </c>
+      <c r="J121" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K121" t="n">
+        <v>0.14</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -19449,13 +19765,13 @@
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="12"/>
-    <col customWidth="1" max="2" min="2" width="12"/>
-    <col customWidth="1" max="3" min="3" width="22"/>
-    <col customWidth="1" max="4" min="4" width="28"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="32" r="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
@@ -19733,10 +20049,13 @@
           <t>Whitefield</t>
         </is>
       </c>
+      <c r="C21" t="n">
+        <v>0.202</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -19749,8 +20068,8 @@
   <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="36"/>
-    <col customWidth="1" max="2" min="2" width="110"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19765,7 +20084,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="2">
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Blank cells</t>
@@ -19777,7 +20096,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="3">
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Digs</t>
@@ -19789,7 +20108,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="4">
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Assists</t>
@@ -19801,7 +20120,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="5">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Attack attempts, Kills, Kill errors</t>
@@ -19813,7 +20132,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="6">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Kill efficiency</t>
@@ -19825,7 +20144,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="7">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Kill efficiency (calculated)</t>
@@ -19837,7 +20156,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="8">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Serve attempts, Aces, Serve errors</t>
@@ -19849,7 +20168,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="9">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Serve rating</t>
@@ -19861,7 +20180,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="10">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Serving scores</t>
@@ -19873,7 +20192,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="11">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Unforced errors</t>
@@ -19885,7 +20204,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="12">
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Stuff blocks</t>
@@ -19897,7 +20216,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="13">
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Block touches</t>
@@ -19909,7 +20228,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="14">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Serve receive rating</t>
@@ -19921,7 +20240,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="15">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Serve receive grades</t>
@@ -19933,7 +20252,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="16">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Freeball attempts / rating / grades</t>
@@ -19945,7 +20264,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="17">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Rotation</t>
@@ -19957,7 +20276,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="18">
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Points scored / against / net</t>
@@ -19969,7 +20288,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="19">
+    <row r="19" ht="32" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Serving by set</t>
@@ -19981,7 +20300,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="20">
+    <row r="20" ht="32" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Team kill efficiency</t>
@@ -19993,7 +20312,7 @@
         </is>
       </c>
     </row>
-    <row customHeight="1" ht="32" r="21">
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Note</t>
@@ -20006,6 +20325,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Drop Bridget from October 7 and fill ratings the sheet left blank.
She did not play that match. October 8 had grades with no rating, so those serves and passes were left out of the averages.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/volleyball_stats.xlsx
+++ b/volleyball_stats.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Player stats" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Rotation stats" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Serving by set" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Matches" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Definitions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player stats" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rotation stats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serving by set" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matches" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Player stats'!$A$1:$X$1</definedName>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X258"/>
+  <dimension ref="A1:X257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5418,6 +5418,9 @@
       <c r="M96" t="n">
         <v>1</v>
       </c>
+      <c r="N96" t="n">
+        <v>0</v>
+      </c>
       <c r="O96" t="inlineStr">
         <is>
           <t>0 0</t>
@@ -13591,14 +13594,14 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Bridget</t>
+          <t>Addy</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F247" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I247" t="n">
         <v>0</v>
@@ -13607,43 +13610,24 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
+        <v>7</v>
+      </c>
+      <c r="L247" t="n">
         <v>1</v>
       </c>
       <c r="M247" t="n">
         <v>1</v>
       </c>
       <c r="N247" t="n">
-        <v>0</v>
+        <v>2.71</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5 0 3 2 3 3 3</t>
         </is>
       </c>
       <c r="P247" t="n">
-        <v>2</v>
-      </c>
-      <c r="S247" t="n">
-        <v>1</v>
-      </c>
-      <c r="T247" t="n">
-        <v>2</v>
-      </c>
-      <c r="U247" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="V247" t="n">
-        <v>1</v>
-      </c>
-      <c r="W247" t="n">
-        <v>3</v>
-      </c>
-      <c r="X247" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="248">
@@ -13657,65 +13641,72 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Addy</t>
-        </is>
-      </c>
-      <c r="D248" t="n">
-        <v>1</v>
-      </c>
-      <c r="F248" t="n">
-        <v>3</v>
-      </c>
-      <c r="I248" t="n">
-        <v>0</v>
-      </c>
-      <c r="J248" t="n">
-        <v>0</v>
-      </c>
-      <c r="K248" t="n">
-        <v>7</v>
-      </c>
-      <c r="L248" t="n">
-        <v>1</v>
-      </c>
-      <c r="M248" t="n">
-        <v>1</v>
-      </c>
-      <c r="N248" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="O248" t="inlineStr">
-        <is>
-          <t>5 0 3 2 3 3 3</t>
-        </is>
-      </c>
-      <c r="P248" t="n">
-        <v>1</v>
+          <t>Emma</t>
+        </is>
+      </c>
+      <c r="S248" t="n">
+        <v>2</v>
+      </c>
+      <c r="T248" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>3 0</t>
+        </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="14" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>First Baptist</t>
+          <t>Whitefield</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Emma</t>
-        </is>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>3</v>
+      </c>
+      <c r="K249" t="n">
+        <v>1</v>
+      </c>
+      <c r="N249" t="n">
+        <v>3</v>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P249" t="n">
+        <v>1</v>
       </c>
       <c r="S249" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="T249" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="U249" t="inlineStr">
         <is>
-          <t>3 0</t>
+          <t>3 0 3 1 2 0 1 1 2 1</t>
+        </is>
+      </c>
+      <c r="V249" t="n">
+        <v>1</v>
+      </c>
+      <c r="W249" t="n">
+        <v>1</v>
+      </c>
+      <c r="X249" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -13730,37 +13721,55 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Annabelle</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="F250" t="n">
+        <v>12</v>
+      </c>
+      <c r="G250" t="n">
+        <v>1</v>
+      </c>
+      <c r="H250" t="n">
+        <v>2</v>
+      </c>
+      <c r="J250" t="n">
+        <v>-0.083</v>
       </c>
       <c r="K250" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="N250" t="n">
+        <v>2.67</v>
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P250" t="n">
-        <v>1</v>
+          <t>3 2 2 3 3 3</t>
+        </is>
       </c>
       <c r="S250" t="n">
-        <v>10</v>
+        <v>3</v>
+      </c>
+      <c r="T250" t="n">
+        <v>2</v>
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>3 0 3 1 2 0 1 1 2 1</t>
+          <t>2 3 1</t>
         </is>
       </c>
       <c r="V250" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="W250" t="n">
+        <v>1.83</v>
       </c>
       <c r="X250" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3 0 2 2 2 2</t>
         </is>
       </c>
     </row>
@@ -13775,46 +13784,44 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Annabelle</t>
+          <t>Nataly</t>
         </is>
       </c>
       <c r="D251" t="n">
         <v>1</v>
       </c>
-      <c r="F251" t="n">
-        <v>12</v>
-      </c>
-      <c r="G251" t="n">
-        <v>1</v>
-      </c>
-      <c r="H251" t="n">
-        <v>2</v>
-      </c>
-      <c r="J251" t="n">
-        <v>-0.083</v>
+      <c r="E251" t="n">
+        <v>4</v>
       </c>
       <c r="K251" t="n">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="L251" t="n">
+        <v>2</v>
+      </c>
+      <c r="M251" t="n">
+        <v>2</v>
+      </c>
+      <c r="N251" t="n">
+        <v>2.6</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>3 2 2 3 3 3</t>
-        </is>
-      </c>
-      <c r="S251" t="n">
-        <v>3</v>
-      </c>
-      <c r="U251" t="inlineStr">
-        <is>
-          <t>2 3 1</t>
-        </is>
+          <t>0 5 5 3 0</t>
+        </is>
+      </c>
+      <c r="P251" t="n">
+        <v>1</v>
       </c>
       <c r="V251" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="W251" t="n">
+        <v>2.5</v>
       </c>
       <c r="X251" t="inlineStr">
         <is>
-          <t>3 0 2 2 2 2</t>
+          <t>2 3</t>
         </is>
       </c>
     </row>
@@ -13829,38 +13836,52 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Nataly</t>
-        </is>
-      </c>
-      <c r="D252" t="n">
-        <v>1</v>
+          <t>Tea</t>
+        </is>
       </c>
       <c r="E252" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="F252" t="n">
+        <v>7</v>
+      </c>
+      <c r="G252" t="n">
+        <v>2</v>
+      </c>
+      <c r="J252" t="n">
+        <v>0.286</v>
       </c>
       <c r="K252" t="n">
-        <v>5</v>
-      </c>
-      <c r="L252" t="n">
-        <v>2</v>
-      </c>
-      <c r="M252" t="n">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="N252" t="n">
+        <v>3</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>0 5 5 3 0</t>
-        </is>
-      </c>
-      <c r="P252" t="n">
-        <v>1</v>
+          <t>3 3</t>
+        </is>
+      </c>
+      <c r="S252" t="n">
+        <v>2</v>
+      </c>
+      <c r="T252" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>3 2</t>
+        </is>
       </c>
       <c r="V252" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="W252" t="n">
+        <v>2.5</v>
       </c>
       <c r="X252" t="inlineStr">
         <is>
-          <t>2 3</t>
+          <t>2 3 3 2</t>
         </is>
       </c>
     </row>
@@ -13875,44 +13896,29 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Tea</t>
-        </is>
-      </c>
-      <c r="E253" t="n">
-        <v>1</v>
+          <t>Cora</t>
+        </is>
       </c>
       <c r="F253" t="n">
         <v>7</v>
       </c>
       <c r="G253" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="H253" t="n">
+        <v>1</v>
       </c>
       <c r="J253" t="n">
-        <v>0.286</v>
-      </c>
-      <c r="K253" t="n">
-        <v>2</v>
-      </c>
-      <c r="O253" t="inlineStr">
-        <is>
-          <t>3 3</t>
-        </is>
-      </c>
-      <c r="S253" t="n">
-        <v>2</v>
-      </c>
-      <c r="U253" t="inlineStr">
-        <is>
-          <t>3 2</t>
-        </is>
-      </c>
-      <c r="V253" t="n">
-        <v>4</v>
-      </c>
-      <c r="X253" t="inlineStr">
-        <is>
-          <t>2 3 3 2</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="P253" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q253" t="n">
+        <v>2</v>
+      </c>
+      <c r="R253" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="254">
@@ -13926,8 +13932,11 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Cora</t>
-        </is>
+          <t>Shiloh</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>6</v>
       </c>
       <c r="F254" t="n">
         <v>7</v>
@@ -13936,19 +13945,46 @@
         <v>1</v>
       </c>
       <c r="H254" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J254" t="n">
-        <v>0</v>
-      </c>
-      <c r="P254" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q254" t="n">
-        <v>2</v>
-      </c>
-      <c r="R254" t="n">
-        <v>2</v>
+        <v>-0.143</v>
+      </c>
+      <c r="K254" t="n">
+        <v>7</v>
+      </c>
+      <c r="L254" t="n">
+        <v>4</v>
+      </c>
+      <c r="N254" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>3 3 5 5 5 5 3</t>
+        </is>
+      </c>
+      <c r="S254" t="n">
+        <v>6</v>
+      </c>
+      <c r="T254" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>2 3 2 1 3 3</t>
+        </is>
+      </c>
+      <c r="V254" t="n">
+        <v>8</v>
+      </c>
+      <c r="W254" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="X254" t="inlineStr">
+        <is>
+          <t>3 3 3 3 3 3 2 3</t>
+        </is>
       </c>
     </row>
     <row r="255">
@@ -13962,11 +13998,8 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Shiloh</t>
-        </is>
-      </c>
-      <c r="D255" t="n">
-        <v>6</v>
+          <t>Agnes</t>
+        </is>
       </c>
       <c r="F255" t="n">
         <v>7</v>
@@ -13980,32 +14013,8 @@
       <c r="J255" t="n">
         <v>-0.143</v>
       </c>
-      <c r="K255" t="n">
-        <v>7</v>
-      </c>
-      <c r="L255" t="n">
-        <v>4</v>
-      </c>
-      <c r="O255" t="inlineStr">
-        <is>
-          <t>3 3 5 5 5 5 3</t>
-        </is>
-      </c>
-      <c r="S255" t="n">
-        <v>6</v>
-      </c>
-      <c r="U255" t="inlineStr">
-        <is>
-          <t>2 3 2 1 3 3</t>
-        </is>
-      </c>
-      <c r="V255" t="n">
-        <v>8</v>
-      </c>
-      <c r="X255" t="inlineStr">
-        <is>
-          <t>3 3 3 3 3 3 2 3</t>
-        </is>
+      <c r="P255" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="256">
@@ -14019,23 +14028,22 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Agnes</t>
-        </is>
-      </c>
-      <c r="F256" t="n">
-        <v>7</v>
-      </c>
-      <c r="G256" t="n">
-        <v>1</v>
-      </c>
-      <c r="H256" t="n">
-        <v>2</v>
-      </c>
-      <c r="J256" t="n">
-        <v>-0.143</v>
-      </c>
-      <c r="P256" t="n">
-        <v>2</v>
+          <t>Addy</t>
+        </is>
+      </c>
+      <c r="K256" t="n">
+        <v>3</v>
+      </c>
+      <c r="L256" t="n">
+        <v>1</v>
+      </c>
+      <c r="N256" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>3 5 3</t>
+        </is>
       </c>
     </row>
     <row r="257">
@@ -14049,42 +14057,19 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Addy</t>
+          <t>Kinley</t>
         </is>
       </c>
       <c r="K257" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L257" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="N257" t="n">
+        <v>4</v>
       </c>
       <c r="O257" t="inlineStr">
-        <is>
-          <t>3 5 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="14" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>Whitefield</t>
-        </is>
-      </c>
-      <c r="C258" t="inlineStr">
-        <is>
-          <t>Kinley</t>
-        </is>
-      </c>
-      <c r="K258" t="n">
-        <v>6</v>
-      </c>
-      <c r="L258" t="n">
-        <v>3</v>
-      </c>
-      <c r="O258" t="inlineStr">
         <is>
           <t>5 5 3 5 3 3</t>
         </is>

</xml_diff>

<commit_message>
Show Bridget's October 7 line from the stat sheet.
That row is on the First Baptist 107 tab, including 3 digs, so the site should keep it.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/volleyball_stats.xlsx
+++ b/volleyball_stats.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Player stats" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Rotation stats" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Serving by set" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Matches" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Definitions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player stats" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rotation stats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Serving by set" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matches" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Player stats'!$A$1:$X$1</definedName>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X267"/>
+  <dimension ref="A1:X268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13594,14 +13594,14 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Addy</t>
+          <t>Bridget</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F247" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I247" t="n">
         <v>0</v>
@@ -13610,24 +13610,43 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
-        <v>7</v>
-      </c>
-      <c r="L247" t="n">
         <v>1</v>
       </c>
       <c r="M247" t="n">
         <v>1</v>
       </c>
       <c r="N247" t="n">
-        <v>2.71</v>
+        <v>0</v>
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>5 0 3 2 3 3 3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P247" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="S247" t="n">
+        <v>1</v>
+      </c>
+      <c r="T247" t="n">
+        <v>2</v>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V247" t="n">
+        <v>1</v>
+      </c>
+      <c r="W247" t="n">
+        <v>3</v>
+      </c>
+      <c r="X247" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="248">
@@ -13641,72 +13660,65 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Emma</t>
-        </is>
-      </c>
-      <c r="S248" t="n">
-        <v>2</v>
-      </c>
-      <c r="T248" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="U248" t="inlineStr">
-        <is>
-          <t>3 0</t>
-        </is>
+          <t>Addy</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>1</v>
+      </c>
+      <c r="F248" t="n">
+        <v>3</v>
+      </c>
+      <c r="I248" t="n">
+        <v>0</v>
+      </c>
+      <c r="J248" t="n">
+        <v>0</v>
+      </c>
+      <c r="K248" t="n">
+        <v>7</v>
+      </c>
+      <c r="L248" t="n">
+        <v>1</v>
+      </c>
+      <c r="M248" t="n">
+        <v>1</v>
+      </c>
+      <c r="N248" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>5 0 3 2 3 3 3</t>
+        </is>
+      </c>
+      <c r="P248" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="14" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Whitefield</t>
+          <t>First Baptist</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Anna</t>
-        </is>
-      </c>
-      <c r="D249" t="n">
-        <v>3</v>
-      </c>
-      <c r="K249" t="n">
-        <v>1</v>
-      </c>
-      <c r="N249" t="n">
-        <v>3</v>
-      </c>
-      <c r="O249" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="P249" t="n">
-        <v>2</v>
+          <t>Emma</t>
+        </is>
       </c>
       <c r="S249" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="T249" t="n">
-        <v>1.53</v>
+        <v>1.5</v>
       </c>
       <c r="U249" t="inlineStr">
         <is>
-          <t>3 0 3 1 2 0 1 1 2 1 2 2 1 2 1 2 2 3 0</t>
-        </is>
-      </c>
-      <c r="V249" t="n">
-        <v>5</v>
-      </c>
-      <c r="W249" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="X249" t="inlineStr">
-        <is>
-          <t>1 2 0 3 2</t>
+          <t>3 0</t>
         </is>
       </c>
     </row>
@@ -13721,64 +13733,46 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Annabelle</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="D250" t="n">
+        <v>3</v>
+      </c>
+      <c r="K250" t="n">
+        <v>1</v>
+      </c>
+      <c r="N250" t="n">
+        <v>3</v>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="P250" t="n">
+        <v>2</v>
+      </c>
+      <c r="S250" t="n">
+        <v>19</v>
+      </c>
+      <c r="T250" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>3 0 3 1 2 0 1 1 2 1 2 2 1 2 1 2 2 3 0</t>
+        </is>
+      </c>
+      <c r="V250" t="n">
         <v>5</v>
       </c>
-      <c r="F250" t="n">
-        <v>15</v>
-      </c>
-      <c r="G250" t="n">
-        <v>1</v>
-      </c>
-      <c r="H250" t="n">
-        <v>2</v>
-      </c>
-      <c r="I250" t="n">
-        <v>-0.067</v>
-      </c>
-      <c r="J250" t="n">
-        <v>-0.067</v>
-      </c>
-      <c r="K250" t="n">
-        <v>13</v>
-      </c>
-      <c r="L250" t="n">
-        <v>3</v>
-      </c>
-      <c r="M250" t="n">
-        <v>1</v>
-      </c>
-      <c r="N250" t="n">
-        <v>3</v>
-      </c>
-      <c r="O250" t="inlineStr">
-        <is>
-          <t>3 2 2 3 3 3 3 0 5 3 5 5 2</t>
-        </is>
-      </c>
-      <c r="S250" t="n">
-        <v>4</v>
-      </c>
-      <c r="T250" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="U250" t="inlineStr">
-        <is>
-          <t>2 3 1 1</t>
-        </is>
-      </c>
-      <c r="V250" t="n">
-        <v>6</v>
-      </c>
       <c r="W250" t="n">
-        <v>1.83</v>
+        <v>1.6</v>
       </c>
       <c r="X250" t="inlineStr">
         <is>
-          <t>3 0 2 2 2 2</t>
+          <t>1 2 0 3 2</t>
         </is>
       </c>
     </row>
@@ -13793,53 +13787,64 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Nataly</t>
+          <t>Annabelle</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>1</v>
-      </c>
-      <c r="E251" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F251" t="n">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="G251" t="n">
+        <v>1</v>
+      </c>
+      <c r="H251" t="n">
+        <v>2</v>
       </c>
       <c r="I251" t="n">
-        <v>0</v>
+        <v>-0.067</v>
       </c>
       <c r="J251" t="n">
-        <v>0</v>
+        <v>-0.067</v>
       </c>
       <c r="K251" t="n">
+        <v>13</v>
+      </c>
+      <c r="L251" t="n">
+        <v>3</v>
+      </c>
+      <c r="M251" t="n">
+        <v>1</v>
+      </c>
+      <c r="N251" t="n">
+        <v>3</v>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>3 2 2 3 3 3 3 0 5 3 5 5 2</t>
+        </is>
+      </c>
+      <c r="S251" t="n">
+        <v>4</v>
+      </c>
+      <c r="T251" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>2 3 1 1</t>
+        </is>
+      </c>
+      <c r="V251" t="n">
         <v>6</v>
       </c>
-      <c r="L251" t="n">
-        <v>2</v>
-      </c>
-      <c r="M251" t="n">
-        <v>2</v>
-      </c>
-      <c r="N251" t="n">
-        <v>2.67</v>
-      </c>
-      <c r="O251" t="inlineStr">
-        <is>
-          <t>0 5 5 3 0 3</t>
-        </is>
-      </c>
-      <c r="P251" t="n">
-        <v>2</v>
-      </c>
-      <c r="V251" t="n">
-        <v>2</v>
-      </c>
       <c r="W251" t="n">
-        <v>2.5</v>
+        <v>1.83</v>
       </c>
       <c r="X251" t="inlineStr">
         <is>
-          <t>2 3</t>
+          <t>3 0 2 2 2 2</t>
         </is>
       </c>
     </row>
@@ -13854,55 +13859,53 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Tea</t>
-        </is>
+          <t>Nataly</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>1</v>
       </c>
       <c r="E252" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F252" t="n">
-        <v>10</v>
-      </c>
-      <c r="G252" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I252" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J252" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="K252" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="L252" t="n">
+        <v>2</v>
+      </c>
+      <c r="M252" t="n">
+        <v>2</v>
       </c>
       <c r="N252" t="n">
-        <v>2.5</v>
+        <v>2.67</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>3 3 1 3</t>
-        </is>
-      </c>
-      <c r="S252" t="n">
-        <v>6</v>
-      </c>
-      <c r="T252" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="U252" t="inlineStr">
-        <is>
-          <t>3 2 1 3 2 3</t>
-        </is>
+          <t>0 5 5 3 0 3</t>
+        </is>
+      </c>
+      <c r="P252" t="n">
+        <v>2</v>
       </c>
       <c r="V252" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W252" t="n">
         <v>2.5</v>
       </c>
       <c r="X252" t="inlineStr">
         <is>
-          <t>2 3 3 2</t>
+          <t>2 3</t>
         </is>
       </c>
     </row>
@@ -13917,32 +13920,56 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Cora</t>
-        </is>
+          <t>Tea</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>1</v>
       </c>
       <c r="F253" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G253" t="n">
-        <v>1</v>
-      </c>
-      <c r="H253" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I253" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J253" t="n">
-        <v>0</v>
-      </c>
-      <c r="P253" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q253" t="n">
-        <v>2</v>
-      </c>
-      <c r="R253" t="n">
-        <v>3</v>
+        <v>0.3</v>
+      </c>
+      <c r="K253" t="n">
+        <v>4</v>
+      </c>
+      <c r="N253" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>3 3 1 3</t>
+        </is>
+      </c>
+      <c r="S253" t="n">
+        <v>6</v>
+      </c>
+      <c r="T253" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>3 2 1 3 2 3</t>
+        </is>
+      </c>
+      <c r="V253" t="n">
+        <v>4</v>
+      </c>
+      <c r="W253" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>2 3 3 2</t>
+        </is>
       </c>
     </row>
     <row r="254">
@@ -13956,65 +13983,32 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Shiloh</t>
-        </is>
-      </c>
-      <c r="D254" t="n">
-        <v>9</v>
+          <t>Cora</t>
+        </is>
       </c>
       <c r="F254" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G254" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H254" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I254" t="n">
-        <v>0.077</v>
+        <v>0</v>
       </c>
       <c r="J254" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="K254" t="n">
-        <v>10</v>
-      </c>
-      <c r="L254" t="n">
-        <v>5</v>
-      </c>
-      <c r="M254" t="n">
-        <v>1</v>
-      </c>
-      <c r="N254" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="O254" t="inlineStr">
-        <is>
-          <t>3 3 5 5 5 5 3 5 2 0</t>
-        </is>
-      </c>
-      <c r="S254" t="n">
-        <v>11</v>
-      </c>
-      <c r="T254" t="n">
-        <v>2.36</v>
-      </c>
-      <c r="U254" t="inlineStr">
-        <is>
-          <t>2 3 2 1 3 3 3 1 2 3 3</t>
-        </is>
-      </c>
-      <c r="V254" t="n">
-        <v>14</v>
-      </c>
-      <c r="W254" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="X254" t="inlineStr">
-        <is>
-          <t>3 3 3 3 3 3 2 3 3 1 3 2 3 2</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="P254" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q254" t="n">
+        <v>2</v>
+      </c>
+      <c r="R254" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="255">
@@ -14028,26 +14022,65 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Agnes</t>
-        </is>
+          <t>Shiloh</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>9</v>
       </c>
       <c r="F255" t="n">
         <v>13</v>
       </c>
       <c r="G255" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H255" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I255" t="n">
-        <v>-0.154</v>
+        <v>0.077</v>
       </c>
       <c r="J255" t="n">
-        <v>-0.154</v>
-      </c>
-      <c r="P255" t="n">
-        <v>2</v>
+        <v>0.077</v>
+      </c>
+      <c r="K255" t="n">
+        <v>10</v>
+      </c>
+      <c r="L255" t="n">
+        <v>5</v>
+      </c>
+      <c r="M255" t="n">
+        <v>1</v>
+      </c>
+      <c r="N255" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>3 3 5 5 5 5 3 5 2 0</t>
+        </is>
+      </c>
+      <c r="S255" t="n">
+        <v>11</v>
+      </c>
+      <c r="T255" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>2 3 2 1 3 3 3 1 2 3 3</t>
+        </is>
+      </c>
+      <c r="V255" t="n">
+        <v>14</v>
+      </c>
+      <c r="W255" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="X255" t="inlineStr">
+        <is>
+          <t>3 3 3 3 3 3 2 3 3 1 3 2 3 2</t>
+        </is>
       </c>
     </row>
     <row r="256">
@@ -14061,28 +14094,26 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Addy</t>
+          <t>Agnes</t>
         </is>
       </c>
       <c r="F256" t="n">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="G256" t="n">
+        <v>2</v>
+      </c>
+      <c r="H256" t="n">
+        <v>4</v>
+      </c>
+      <c r="I256" t="n">
+        <v>-0.154</v>
       </c>
       <c r="J256" t="n">
-        <v>0</v>
-      </c>
-      <c r="K256" t="n">
-        <v>5</v>
-      </c>
-      <c r="L256" t="n">
-        <v>2</v>
-      </c>
-      <c r="N256" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="O256" t="inlineStr">
-        <is>
-          <t>3 5 3 2 5</t>
-        </is>
+        <v>-0.154</v>
+      </c>
+      <c r="P256" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="257">
@@ -14096,24 +14127,27 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Kinley</t>
-        </is>
+          <t>Addy</t>
+        </is>
+      </c>
+      <c r="F257" t="n">
+        <v>1</v>
+      </c>
+      <c r="J257" t="n">
+        <v>0</v>
       </c>
       <c r="K257" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="L257" t="n">
-        <v>6</v>
-      </c>
-      <c r="M257" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N257" t="n">
-        <v>3.58</v>
+        <v>3.6</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>5 5 3 5 3 3 5 5 0 5 2 2</t>
+          <t>3 5 3 2 5</t>
         </is>
       </c>
     </row>
@@ -14128,58 +14162,55 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Corena</t>
-        </is>
-      </c>
-      <c r="D258" t="n">
-        <v>1</v>
-      </c>
-      <c r="E258" t="n">
-        <v>2</v>
-      </c>
-      <c r="F258" t="n">
-        <v>1</v>
-      </c>
-      <c r="J258" t="n">
-        <v>0</v>
-      </c>
-      <c r="P258" t="n">
-        <v>1</v>
+          <t>Kinley</t>
+        </is>
+      </c>
+      <c r="K258" t="n">
+        <v>12</v>
+      </c>
+      <c r="L258" t="n">
+        <v>6</v>
+      </c>
+      <c r="M258" t="n">
+        <v>1</v>
+      </c>
+      <c r="N258" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>5 5 3 5 3 3 5 5 0 5 2 2</t>
+        </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Heritage</t>
+          <t>Whitefield</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Tea</t>
-        </is>
+          <t>Corena</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>1</v>
+      </c>
+      <c r="E259" t="n">
+        <v>2</v>
       </c>
       <c r="F259" t="n">
         <v>1</v>
       </c>
-      <c r="G259" t="n">
-        <v>1</v>
-      </c>
       <c r="J259" t="n">
-        <v>1</v>
-      </c>
-      <c r="S259" t="n">
-        <v>3</v>
-      </c>
-      <c r="T259" t="n">
-        <v>2</v>
-      </c>
-      <c r="U259" t="inlineStr">
-        <is>
-          <t>1 3 2</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="P259" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="260">
@@ -14193,23 +14224,28 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Annabelle</t>
-        </is>
-      </c>
-      <c r="D260" t="n">
-        <v>1</v>
-      </c>
-      <c r="E260" t="n">
-        <v>1</v>
+          <t>Tea</t>
+        </is>
       </c>
       <c r="F260" t="n">
         <v>1</v>
       </c>
-      <c r="H260" t="n">
+      <c r="G260" t="n">
         <v>1</v>
       </c>
       <c r="J260" t="n">
-        <v>-1</v>
+        <v>1</v>
+      </c>
+      <c r="S260" t="n">
+        <v>3</v>
+      </c>
+      <c r="T260" t="n">
+        <v>2</v>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>1 3 2</t>
+        </is>
       </c>
     </row>
     <row r="261">
@@ -14223,17 +14259,23 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Cora</t>
-        </is>
+          <t>Annabelle</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>1</v>
+      </c>
+      <c r="E261" t="n">
+        <v>1</v>
       </c>
       <c r="F261" t="n">
-        <v>3</v>
-      </c>
-      <c r="G261" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="H261" t="n">
+        <v>1</v>
       </c>
       <c r="J261" t="n">
-        <v>0.667</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="262">
@@ -14247,44 +14289,17 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Shiloh</t>
-        </is>
-      </c>
-      <c r="K262" t="n">
-        <v>10</v>
-      </c>
-      <c r="L262" t="n">
-        <v>1</v>
-      </c>
-      <c r="N262" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="O262" t="inlineStr">
-        <is>
-          <t>3 5 3 3 3 3 2 1 3 3</t>
-        </is>
-      </c>
-      <c r="S262" t="n">
-        <v>2</v>
-      </c>
-      <c r="T262" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="U262" t="inlineStr">
-        <is>
-          <t>1 2</t>
-        </is>
-      </c>
-      <c r="V262" t="n">
-        <v>1</v>
-      </c>
-      <c r="W262" t="n">
-        <v>2</v>
-      </c>
-      <c r="X262" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>3</v>
+      </c>
+      <c r="G262" t="n">
+        <v>2</v>
+      </c>
+      <c r="J262" t="n">
+        <v>0.667</v>
       </c>
     </row>
     <row r="263">
@@ -14298,7 +14313,21 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Shiloh</t>
+        </is>
+      </c>
+      <c r="K263" t="n">
+        <v>10</v>
+      </c>
+      <c r="L263" t="n">
+        <v>1</v>
+      </c>
+      <c r="N263" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>3 5 3 3 3 3 2 1 3 3</t>
         </is>
       </c>
       <c r="S263" t="n">
@@ -14309,18 +14338,18 @@
       </c>
       <c r="U263" t="inlineStr">
         <is>
-          <t>0 3</t>
+          <t>1 2</t>
         </is>
       </c>
       <c r="V263" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W263" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="X263" t="inlineStr">
         <is>
-          <t>3 2</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -14335,14 +14364,30 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Nataly</t>
-        </is>
-      </c>
-      <c r="E264" t="n">
-        <v>1</v>
-      </c>
-      <c r="P264" t="n">
-        <v>1</v>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="S264" t="n">
+        <v>2</v>
+      </c>
+      <c r="T264" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="U264" t="inlineStr">
+        <is>
+          <t>0 3</t>
+        </is>
+      </c>
+      <c r="V264" t="n">
+        <v>2</v>
+      </c>
+      <c r="W264" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="X264" t="inlineStr">
+        <is>
+          <t>3 2</t>
+        </is>
       </c>
     </row>
     <row r="265">
@@ -14356,22 +14401,14 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Kinley</t>
-        </is>
-      </c>
-      <c r="K265" t="n">
-        <v>1</v>
-      </c>
-      <c r="M265" t="n">
-        <v>1</v>
-      </c>
-      <c r="N265" t="n">
-        <v>0</v>
-      </c>
-      <c r="O265" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>Nataly</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>1</v>
+      </c>
+      <c r="P265" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="266">
@@ -14385,17 +14422,22 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Agnes</t>
-        </is>
-      </c>
-      <c r="F266" t="n">
-        <v>2</v>
-      </c>
-      <c r="H266" t="n">
-        <v>1</v>
-      </c>
-      <c r="J266" t="n">
-        <v>-0.5</v>
+          <t>Kinley</t>
+        </is>
+      </c>
+      <c r="K266" t="n">
+        <v>1</v>
+      </c>
+      <c r="M266" t="n">
+        <v>1</v>
+      </c>
+      <c r="N266" t="n">
+        <v>0</v>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
     </row>
     <row r="267">
@@ -14409,16 +14451,40 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
+          <t>Agnes</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>2</v>
+      </c>
+      <c r="H267" t="n">
+        <v>1</v>
+      </c>
+      <c r="J267" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="14" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
           <t>Addy</t>
         </is>
       </c>
-      <c r="D267" t="n">
-        <v>1</v>
-      </c>
-      <c r="F267" t="n">
-        <v>2</v>
-      </c>
-      <c r="J267" t="n">
+      <c r="D268" t="n">
+        <v>1</v>
+      </c>
+      <c r="F268" t="n">
+        <v>2</v>
+      </c>
+      <c r="J268" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Calculate ratings from the recorded grades.
Serve, receive, and freeball ratings are the sum of the grades divided by the attempts. The typed rating cell is no longer used.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/volleyball_stats.xlsx
+++ b/volleyball_stats.xlsx
@@ -665,7 +665,7 @@
         <v>7</v>
       </c>
       <c r="T2" t="n">
-        <v>0.71</v>
+        <v>0.714</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -715,7 +715,7 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>3.89</v>
+        <v>3.895</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -729,7 +729,7 @@
         <v>11</v>
       </c>
       <c r="T3" t="n">
-        <v>1.67</v>
+        <v>1.636</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
         <v>1</v>
       </c>
       <c r="N4" t="n">
-        <v>3.67</v>
+        <v>3.636</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         <v>3</v>
       </c>
       <c r="T6" t="n">
-        <v>1.33</v>
+        <v>1.333</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         <v>2</v>
       </c>
       <c r="N7" t="n">
-        <v>3.29</v>
+        <v>3.286</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         <v>17</v>
       </c>
       <c r="T10" t="n">
-        <v>1.59</v>
+        <v>1.706</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1224,7 +1224,7 @@
         <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>2.78</v>
+        <v>2.783</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         <v>7</v>
       </c>
       <c r="W14" t="n">
-        <v>2.29</v>
+        <v>2.286</v>
       </c>
       <c r="X14" t="inlineStr">
         <is>
@@ -1287,7 +1287,7 @@
         <v>2</v>
       </c>
       <c r="N15" t="n">
-        <v>2.92</v>
+        <v>2.923</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1301,7 +1301,7 @@
         <v>3</v>
       </c>
       <c r="W15" t="n">
-        <v>2.67</v>
+        <v>2.667</v>
       </c>
       <c r="X15" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         <v>19</v>
       </c>
       <c r="T16" t="n">
-        <v>1.37</v>
+        <v>1.368</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
         <v>13</v>
       </c>
       <c r="T17" t="n">
-        <v>1.77</v>
+        <v>1.769</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -1477,7 +1477,7 @@
         <v>3</v>
       </c>
       <c r="N18" t="n">
-        <v>2.59</v>
+        <v>2.588</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
         <v>11</v>
       </c>
       <c r="T18" t="n">
-        <v>1.09</v>
+        <v>1.091</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
         <v>5</v>
       </c>
       <c r="N19" t="n">
-        <v>2.67</v>
+        <v>2.667</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1787,7 +1787,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>1 0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
         <v>22</v>
       </c>
       <c r="T26" t="n">
-        <v>1.36</v>
+        <v>1.364</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         <v>3</v>
       </c>
       <c r="N27" t="n">
-        <v>3.29</v>
+        <v>3.286</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>3.06</v>
+        <v>3.056</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2007,7 +2007,7 @@
         <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>1.86</v>
+        <v>1.857</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>7</v>
       </c>
       <c r="T29" t="n">
-        <v>1.71</v>
+        <v>1.714</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>2</v>
       </c>
       <c r="N30" t="n">
-        <v>1.13</v>
+        <v>1.125</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v>3</v>
       </c>
       <c r="T33" t="n">
-        <v>0.67</v>
+        <v>0.667</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         <v>2</v>
       </c>
       <c r="N36" t="n">
-        <v>2.31</v>
+        <v>2.312</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         <v>21</v>
       </c>
       <c r="T36" t="n">
-        <v>1.62</v>
+        <v>1.619</v>
       </c>
       <c r="U36" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
         <v>7</v>
       </c>
       <c r="W36" t="n">
-        <v>2.57</v>
+        <v>2.571</v>
       </c>
       <c r="X36" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
         <v>15</v>
       </c>
       <c r="T38" t="n">
-        <v>1.87</v>
+        <v>1.867</v>
       </c>
       <c r="U38" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
         <v>7</v>
       </c>
       <c r="W38" t="n">
-        <v>2.29</v>
+        <v>2.286</v>
       </c>
       <c r="X38" t="inlineStr">
         <is>
@@ -2512,7 +2512,7 @@
         <v>11</v>
       </c>
       <c r="T39" t="n">
-        <v>1.45</v>
+        <v>1.455</v>
       </c>
       <c r="U39" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         <v>1</v>
       </c>
       <c r="W39" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="X39" t="inlineStr">
         <is>
@@ -2576,7 +2576,7 @@
         <v>1</v>
       </c>
       <c r="N40" t="n">
-        <v>2.91</v>
+        <v>2.909</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -2642,7 +2642,7 @@
         <v>2</v>
       </c>
       <c r="N41" t="n">
-        <v>2.36</v>
+        <v>2.364</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -2714,7 +2714,7 @@
         <v>9</v>
       </c>
       <c r="T42" t="n">
-        <v>1.11</v>
+        <v>1.111</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
@@ -3086,7 +3086,7 @@
         <v>16</v>
       </c>
       <c r="T50" t="n">
-        <v>1.56</v>
+        <v>1.562</v>
       </c>
       <c r="U50" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
         <v>7</v>
       </c>
       <c r="W50" t="n">
-        <v>2.86</v>
+        <v>2.857</v>
       </c>
       <c r="X50" t="inlineStr">
         <is>
@@ -3147,7 +3147,7 @@
         <v>2</v>
       </c>
       <c r="N51" t="n">
-        <v>2.77</v>
+        <v>2.769</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -3208,7 +3208,7 @@
         <v>1</v>
       </c>
       <c r="N52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -3312,7 +3312,7 @@
         <v>2</v>
       </c>
       <c r="N54" t="n">
-        <v>2.36</v>
+        <v>2.364</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -3326,7 +3326,7 @@
         <v>6</v>
       </c>
       <c r="T54" t="n">
-        <v>1.17</v>
+        <v>1.5</v>
       </c>
       <c r="U54" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
         <v>6</v>
       </c>
       <c r="W54" t="n">
-        <v>1.5</v>
+        <v>1.833</v>
       </c>
       <c r="X54" t="inlineStr">
         <is>
@@ -3401,7 +3401,7 @@
         <v>9</v>
       </c>
       <c r="T55" t="n">
-        <v>1.44</v>
+        <v>1.444</v>
       </c>
       <c r="U55" t="inlineStr">
         <is>
@@ -3554,7 +3554,7 @@
         <v>1</v>
       </c>
       <c r="N58" t="n">
-        <v>1.67</v>
+        <v>1.667</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
         <v>11</v>
       </c>
       <c r="N64" t="n">
-        <v>2.84</v>
+        <v>2.844</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -3819,7 +3819,7 @@
         <v>14</v>
       </c>
       <c r="T64" t="n">
-        <v>1.57</v>
+        <v>1.571</v>
       </c>
       <c r="U64" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
         <v>9</v>
       </c>
       <c r="W64" t="n">
-        <v>2.56</v>
+        <v>2.556</v>
       </c>
       <c r="X64" t="inlineStr">
         <is>
@@ -3883,7 +3883,7 @@
         <v>9</v>
       </c>
       <c r="N65" t="n">
-        <v>2.1</v>
+        <v>2.095</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -3939,7 +3939,7 @@
         <v>3</v>
       </c>
       <c r="N66" t="n">
-        <v>2.63</v>
+        <v>2.632</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -3964,7 +3964,7 @@
         <v>3</v>
       </c>
       <c r="W66" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="X66" t="inlineStr">
         <is>
@@ -4014,7 +4014,7 @@
         <v>3</v>
       </c>
       <c r="N67" t="n">
-        <v>2.38</v>
+        <v>2.385</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -4107,7 +4107,7 @@
         <v>3</v>
       </c>
       <c r="N69" t="n">
-        <v>2.38</v>
+        <v>2.385</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -4121,7 +4121,7 @@
         <v>16</v>
       </c>
       <c r="T69" t="n">
-        <v>1.69</v>
+        <v>1.688</v>
       </c>
       <c r="U69" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v>3</v>
       </c>
       <c r="N71" t="n">
-        <v>2.36</v>
+        <v>2.375</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -4209,7 +4209,7 @@
         <v>24</v>
       </c>
       <c r="T71" t="n">
-        <v>2.04</v>
+        <v>2.042</v>
       </c>
       <c r="U71" t="inlineStr">
         <is>
@@ -4442,7 +4442,7 @@
         <v>2</v>
       </c>
       <c r="N76" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -4635,7 +4635,7 @@
         <v>3</v>
       </c>
       <c r="T79" t="n">
-        <v>1.667</v>
+        <v>1.333</v>
       </c>
       <c r="U79" t="inlineStr">
         <is>
@@ -4687,7 +4687,7 @@
         <v>2</v>
       </c>
       <c r="N80" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -4930,7 +4930,7 @@
       </c>
       <c r="U86" t="inlineStr">
         <is>
-          <t>2 0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="X91" t="inlineStr">
         <is>
-          <t>1 0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="U92" t="inlineStr">
         <is>
-          <t>1 0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="V92" t="n">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>0 0</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
         <v>2</v>
       </c>
       <c r="N97" t="n">
-        <v>3.14</v>
+        <v>3.143</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
         <v>8</v>
       </c>
       <c r="W97" t="n">
-        <v>1.86</v>
+        <v>1.875</v>
       </c>
       <c r="X97" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
         <v>2</v>
       </c>
       <c r="N98" t="n">
-        <v>2.31</v>
+        <v>2.308</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -5537,7 +5537,7 @@
         <v>27</v>
       </c>
       <c r="T98" t="n">
-        <v>2.19</v>
+        <v>2.148</v>
       </c>
       <c r="U98" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
         <v>9</v>
       </c>
       <c r="W98" t="n">
-        <v>2.56</v>
+        <v>2.556</v>
       </c>
       <c r="X98" t="inlineStr">
         <is>
@@ -5595,7 +5595,7 @@
         <v>3</v>
       </c>
       <c r="N99" t="n">
-        <v>3.33</v>
+        <v>3.333</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -5609,7 +5609,7 @@
         <v>7</v>
       </c>
       <c r="T99" t="n">
-        <v>0.86</v>
+        <v>0.857</v>
       </c>
       <c r="U99" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
         <v>5</v>
       </c>
       <c r="N100" t="n">
-        <v>1.76</v>
+        <v>2</v>
       </c>
       <c r="O100" t="inlineStr">
         <is>
@@ -5751,7 +5751,7 @@
         <v>7</v>
       </c>
       <c r="N101" t="n">
-        <v>2.43</v>
+        <v>2.429</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -5771,7 +5771,7 @@
         <v>13</v>
       </c>
       <c r="T101" t="n">
-        <v>1.69</v>
+        <v>1.692</v>
       </c>
       <c r="U101" t="inlineStr">
         <is>
@@ -5876,7 +5876,7 @@
         <v>1</v>
       </c>
       <c r="N103" t="n">
-        <v>2.44</v>
+        <v>2.444</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -5896,7 +5896,7 @@
         <v>3</v>
       </c>
       <c r="T103" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="U103" t="inlineStr">
         <is>
@@ -5957,7 +5957,7 @@
         <v>2</v>
       </c>
       <c r="N104" t="n">
-        <v>2.18</v>
+        <v>2.409</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -6015,7 +6015,7 @@
         <v>1</v>
       </c>
       <c r="N105" t="n">
-        <v>1.56</v>
+        <v>1.556</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -6029,7 +6029,7 @@
         <v>16</v>
       </c>
       <c r="T105" t="n">
-        <v>1.06</v>
+        <v>1.062</v>
       </c>
       <c r="U105" t="inlineStr">
         <is>
@@ -6203,7 +6203,7 @@
         <v>3</v>
       </c>
       <c r="N108" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="O108" t="inlineStr">
         <is>
@@ -6292,7 +6292,7 @@
         <v>15</v>
       </c>
       <c r="T109" t="n">
-        <v>1.53</v>
+        <v>1.533</v>
       </c>
       <c r="U109" t="inlineStr">
         <is>
@@ -6303,7 +6303,7 @@
         <v>3</v>
       </c>
       <c r="W109" t="n">
-        <v>2.67</v>
+        <v>2.667</v>
       </c>
       <c r="X109" t="inlineStr">
         <is>
@@ -6411,7 +6411,7 @@
         <v>1</v>
       </c>
       <c r="N111" t="n">
-        <v>1.89</v>
+        <v>1.889</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -6550,7 +6550,7 @@
         <v>1</v>
       </c>
       <c r="N114" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
@@ -6564,7 +6564,7 @@
         <v>8</v>
       </c>
       <c r="T114" t="n">
-        <v>1</v>
+        <v>1.125</v>
       </c>
       <c r="U114" t="inlineStr">
         <is>
@@ -6628,7 +6628,7 @@
         <v>1</v>
       </c>
       <c r="N115" t="n">
-        <v>3.08</v>
+        <v>3.077</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
@@ -6642,7 +6642,7 @@
         <v>3</v>
       </c>
       <c r="T115" t="n">
-        <v>2.67</v>
+        <v>2.667</v>
       </c>
       <c r="U115" t="inlineStr">
         <is>
@@ -6653,7 +6653,7 @@
         <v>7</v>
       </c>
       <c r="W115" t="n">
-        <v>2.71</v>
+        <v>2.429</v>
       </c>
       <c r="X115" t="inlineStr">
         <is>
@@ -6706,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="N116" t="n">
-        <v>2.78</v>
+        <v>2.739</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
@@ -6731,7 +6731,7 @@
         <v>13</v>
       </c>
       <c r="W116" t="n">
-        <v>2.31</v>
+        <v>2.308</v>
       </c>
       <c r="X116" t="inlineStr">
         <is>
@@ -6781,7 +6781,7 @@
         <v>2</v>
       </c>
       <c r="N117" t="n">
-        <v>2.36</v>
+        <v>2.375</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
@@ -6795,7 +6795,7 @@
         <v>11</v>
       </c>
       <c r="T117" t="n">
-        <v>1.27</v>
+        <v>1.273</v>
       </c>
       <c r="U117" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v>7</v>
       </c>
       <c r="T120" t="n">
-        <v>2.29</v>
+        <v>2.286</v>
       </c>
       <c r="U120" t="inlineStr">
         <is>
@@ -7000,7 +7000,7 @@
         <v>1</v>
       </c>
       <c r="N121" t="n">
-        <v>3.33</v>
+        <v>3.333</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
@@ -7326,7 +7326,7 @@
         <v>3</v>
       </c>
       <c r="W128" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="X128" t="inlineStr">
         <is>
@@ -7376,7 +7376,7 @@
         <v>2</v>
       </c>
       <c r="N129" t="n">
-        <v>2.94</v>
+        <v>2.938</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
@@ -7390,7 +7390,7 @@
         <v>7</v>
       </c>
       <c r="T129" t="n">
-        <v>1.57</v>
+        <v>1.571</v>
       </c>
       <c r="U129" t="inlineStr">
         <is>
@@ -7401,7 +7401,7 @@
         <v>9</v>
       </c>
       <c r="W129" t="n">
-        <v>2.56</v>
+        <v>2.556</v>
       </c>
       <c r="X129" t="inlineStr">
         <is>
@@ -7451,7 +7451,7 @@
         <v>2</v>
       </c>
       <c r="N130" t="n">
-        <v>3.47</v>
+        <v>3.474</v>
       </c>
       <c r="O130" t="inlineStr">
         <is>
@@ -7465,7 +7465,7 @@
         <v>7</v>
       </c>
       <c r="T130" t="n">
-        <v>1.14</v>
+        <v>1.143</v>
       </c>
       <c r="U130" t="inlineStr">
         <is>
@@ -7540,7 +7540,7 @@
         <v>13</v>
       </c>
       <c r="T131" t="n">
-        <v>1.15</v>
+        <v>1.154</v>
       </c>
       <c r="U131" t="inlineStr">
         <is>
@@ -7551,7 +7551,7 @@
         <v>8</v>
       </c>
       <c r="W131" t="n">
-        <v>2.13</v>
+        <v>2.125</v>
       </c>
       <c r="X131" t="inlineStr">
         <is>
@@ -7583,7 +7583,7 @@
         <v>4</v>
       </c>
       <c r="N132" t="n">
-        <v>2.31</v>
+        <v>2.308</v>
       </c>
       <c r="O132" t="inlineStr">
         <is>
@@ -7679,7 +7679,7 @@
         <v>2</v>
       </c>
       <c r="N134" t="n">
-        <v>3.08</v>
+        <v>3.083</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
@@ -7837,7 +7837,7 @@
         <v>2</v>
       </c>
       <c r="N137" t="n">
-        <v>2.17</v>
+        <v>2.167</v>
       </c>
       <c r="O137" t="inlineStr">
         <is>
@@ -7851,7 +7851,7 @@
         <v>24</v>
       </c>
       <c r="T137" t="n">
-        <v>1.92</v>
+        <v>1.917</v>
       </c>
       <c r="U137" t="inlineStr">
         <is>
@@ -7915,7 +7915,7 @@
         <v>1</v>
       </c>
       <c r="N138" t="n">
-        <v>3.42</v>
+        <v>3.419</v>
       </c>
       <c r="O138" t="inlineStr">
         <is>
@@ -7929,7 +7929,7 @@
         <v>14</v>
       </c>
       <c r="T138" t="n">
-        <v>1.64</v>
+        <v>1.643</v>
       </c>
       <c r="U138" t="inlineStr">
         <is>
@@ -7940,7 +7940,7 @@
         <v>21</v>
       </c>
       <c r="W138" t="n">
-        <v>2.49</v>
+        <v>2.429</v>
       </c>
       <c r="X138" t="inlineStr">
         <is>
@@ -7993,7 +7993,7 @@
         <v>5</v>
       </c>
       <c r="N139" t="n">
-        <v>2.07</v>
+        <v>2.067</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
@@ -8010,7 +8010,7 @@
         <v>13</v>
       </c>
       <c r="T139" t="n">
-        <v>1.54</v>
+        <v>1.538</v>
       </c>
       <c r="U139" t="inlineStr">
         <is>
@@ -8021,7 +8021,7 @@
         <v>8</v>
       </c>
       <c r="W139" t="n">
-        <v>2.13</v>
+        <v>2.125</v>
       </c>
       <c r="X139" t="inlineStr">
         <is>
@@ -8155,7 +8155,7 @@
         <v>2</v>
       </c>
       <c r="N142" t="n">
-        <v>2.94</v>
+        <v>2.944</v>
       </c>
       <c r="O142" t="inlineStr">
         <is>
@@ -8169,7 +8169,7 @@
         <v>14</v>
       </c>
       <c r="T142" t="n">
-        <v>1.93</v>
+        <v>1.929</v>
       </c>
       <c r="U142" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
         <v>14</v>
       </c>
       <c r="T143" t="n">
-        <v>1.64</v>
+        <v>1.643</v>
       </c>
       <c r="U143" t="inlineStr">
         <is>
@@ -8237,7 +8237,7 @@
         <v>9</v>
       </c>
       <c r="W143" t="n">
-        <v>2.67</v>
+        <v>2.667</v>
       </c>
       <c r="X143" t="inlineStr">
         <is>
@@ -8337,7 +8337,7 @@
         <v>7</v>
       </c>
       <c r="W145" t="n">
-        <v>2.14</v>
+        <v>2.143</v>
       </c>
       <c r="X145" t="inlineStr">
         <is>
@@ -8405,7 +8405,7 @@
         <v>3</v>
       </c>
       <c r="N147" t="n">
-        <v>1.53</v>
+        <v>1.533</v>
       </c>
       <c r="O147" t="inlineStr">
         <is>
@@ -8461,7 +8461,7 @@
         <v>2</v>
       </c>
       <c r="N148" t="n">
-        <v>2.47</v>
+        <v>2.471</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
@@ -8475,7 +8475,7 @@
         <v>22</v>
       </c>
       <c r="T148" t="n">
-        <v>2.32</v>
+        <v>2.318</v>
       </c>
       <c r="U148" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>23</v>
       </c>
       <c r="W148" t="n">
-        <v>2.48</v>
+        <v>2.478</v>
       </c>
       <c r="X148" t="inlineStr">
         <is>
@@ -8529,7 +8529,7 @@
         <v>17</v>
       </c>
       <c r="T149" t="n">
-        <v>2.24</v>
+        <v>2.235</v>
       </c>
       <c r="U149" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
         <v>13</v>
       </c>
       <c r="W150" t="n">
-        <v>2.15</v>
+        <v>2.154</v>
       </c>
       <c r="X150" t="inlineStr">
         <is>
@@ -8665,7 +8665,7 @@
         <v>5</v>
       </c>
       <c r="N151" t="n">
-        <v>2.31</v>
+        <v>2.312</v>
       </c>
       <c r="O151" t="inlineStr">
         <is>
@@ -8682,7 +8682,7 @@
         <v>13</v>
       </c>
       <c r="T151" t="n">
-        <v>1.59</v>
+        <v>1.538</v>
       </c>
       <c r="U151" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
         <v>7</v>
       </c>
       <c r="W152" t="n">
-        <v>1.86</v>
+        <v>1.857</v>
       </c>
       <c r="X152" t="inlineStr">
         <is>
@@ -8795,7 +8795,7 @@
         <v>1</v>
       </c>
       <c r="N153" t="n">
-        <v>1.67</v>
+        <v>1.667</v>
       </c>
       <c r="O153" t="inlineStr">
         <is>
@@ -8856,7 +8856,7 @@
         <v>3</v>
       </c>
       <c r="N154" t="n">
-        <v>2.56</v>
+        <v>2.556</v>
       </c>
       <c r="O154" t="inlineStr">
         <is>
@@ -8867,7 +8867,7 @@
         <v>12</v>
       </c>
       <c r="T154" t="n">
-        <v>1.67</v>
+        <v>1.667</v>
       </c>
       <c r="U154" t="inlineStr">
         <is>
@@ -8961,7 +8961,7 @@
         <v>1</v>
       </c>
       <c r="N156" t="n">
-        <v>2.45</v>
+        <v>2.455</v>
       </c>
       <c r="O156" t="inlineStr">
         <is>
@@ -9049,7 +9049,7 @@
         <v>1</v>
       </c>
       <c r="N159" t="n">
-        <v>1.36</v>
+        <v>1.375</v>
       </c>
       <c r="O159" t="inlineStr">
         <is>
@@ -9060,7 +9060,7 @@
         <v>24</v>
       </c>
       <c r="T159" t="n">
-        <v>1.38</v>
+        <v>1.375</v>
       </c>
       <c r="U159" t="inlineStr">
         <is>
@@ -9071,7 +9071,7 @@
         <v>6</v>
       </c>
       <c r="W159" t="n">
-        <v>2.17</v>
+        <v>2.167</v>
       </c>
       <c r="X159" t="inlineStr">
         <is>
@@ -9159,7 +9159,7 @@
         <v>18</v>
       </c>
       <c r="T161" t="n">
-        <v>1.39</v>
+        <v>1.389</v>
       </c>
       <c r="U161" t="inlineStr">
         <is>
@@ -9223,7 +9223,7 @@
         <v>5</v>
       </c>
       <c r="N162" t="n">
-        <v>2.17</v>
+        <v>2.167</v>
       </c>
       <c r="O162" t="inlineStr">
         <is>
@@ -9237,7 +9237,7 @@
         <v>11</v>
       </c>
       <c r="T162" t="n">
-        <v>1.27</v>
+        <v>1.273</v>
       </c>
       <c r="U162" t="inlineStr">
         <is>
@@ -9248,7 +9248,7 @@
         <v>7</v>
       </c>
       <c r="W162" t="n">
-        <v>2.57</v>
+        <v>2.571</v>
       </c>
       <c r="X162" t="inlineStr">
         <is>
@@ -9298,7 +9298,7 @@
         <v>2</v>
       </c>
       <c r="N163" t="n">
-        <v>2.18</v>
+        <v>2.182</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
@@ -9312,7 +9312,7 @@
         <v>22</v>
       </c>
       <c r="T163" t="n">
-        <v>1.59</v>
+        <v>1.591</v>
       </c>
       <c r="U163" t="inlineStr">
         <is>
@@ -9414,7 +9414,7 @@
         <v>4</v>
       </c>
       <c r="N165" t="n">
-        <v>2.31</v>
+        <v>2.312</v>
       </c>
       <c r="O165" t="inlineStr">
         <is>
@@ -9655,7 +9655,7 @@
         <v>26</v>
       </c>
       <c r="T170" t="n">
-        <v>1.73</v>
+        <v>1.731</v>
       </c>
       <c r="U170" t="inlineStr">
         <is>
@@ -9713,7 +9713,7 @@
         <v>2</v>
       </c>
       <c r="N171" t="n">
-        <v>2.82</v>
+        <v>2.818</v>
       </c>
       <c r="O171" t="inlineStr">
         <is>
@@ -9727,7 +9727,7 @@
         <v>19</v>
       </c>
       <c r="T171" t="n">
-        <v>1.59</v>
+        <v>1.579</v>
       </c>
       <c r="U171" t="inlineStr">
         <is>
@@ -9880,7 +9880,7 @@
         <v>10</v>
       </c>
       <c r="T173" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="U173" t="inlineStr">
         <is>
@@ -9923,7 +9923,7 @@
         <v>1</v>
       </c>
       <c r="N174" t="n">
-        <v>2.67</v>
+        <v>2.667</v>
       </c>
       <c r="O174" t="inlineStr">
         <is>
@@ -10285,7 +10285,7 @@
         <v>3</v>
       </c>
       <c r="N183" t="n">
-        <v>3.11</v>
+        <v>3.105</v>
       </c>
       <c r="O183" t="inlineStr">
         <is>
@@ -10402,7 +10402,7 @@
         <v>2</v>
       </c>
       <c r="N185" t="n">
-        <v>3.05</v>
+        <v>2.8</v>
       </c>
       <c r="O185" t="inlineStr">
         <is>
@@ -10416,7 +10416,7 @@
         <v>17</v>
       </c>
       <c r="T185" t="n">
-        <v>1.59</v>
+        <v>1.588</v>
       </c>
       <c r="U185" t="inlineStr">
         <is>
@@ -10427,7 +10427,7 @@
         <v>6</v>
       </c>
       <c r="W185" t="n">
-        <v>2.17</v>
+        <v>2.167</v>
       </c>
       <c r="X185" t="inlineStr">
         <is>
@@ -10496,7 +10496,7 @@
         <v>3</v>
       </c>
       <c r="W186" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="X186" t="inlineStr">
         <is>
@@ -10594,7 +10594,7 @@
         <v>4</v>
       </c>
       <c r="W188" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="X188" t="inlineStr">
         <is>
@@ -10688,7 +10688,7 @@
         <v>2</v>
       </c>
       <c r="N190" t="n">
-        <v>3.42</v>
+        <v>3.417</v>
       </c>
       <c r="O190" t="inlineStr">
         <is>
@@ -10826,7 +10826,7 @@
         <v>4</v>
       </c>
       <c r="N193" t="n">
-        <v>1.67</v>
+        <v>1.667</v>
       </c>
       <c r="O193" t="inlineStr">
         <is>
@@ -10840,7 +10840,7 @@
         <v>7</v>
       </c>
       <c r="T193" t="n">
-        <v>0.86</v>
+        <v>0.857</v>
       </c>
       <c r="U193" t="inlineStr">
         <is>
@@ -10887,7 +10887,7 @@
         <v>8</v>
       </c>
       <c r="N194" t="n">
-        <v>3.87</v>
+        <v>3.867</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
@@ -10901,7 +10901,7 @@
         <v>15</v>
       </c>
       <c r="T194" t="n">
-        <v>1.53</v>
+        <v>1.533</v>
       </c>
       <c r="U194" t="inlineStr">
         <is>
@@ -10947,7 +10947,7 @@
         <v>2</v>
       </c>
       <c r="N195" t="n">
-        <v>1.86</v>
+        <v>1.875</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
         <v>8</v>
       </c>
       <c r="T195" t="n">
-        <v>1.63</v>
+        <v>1.625</v>
       </c>
       <c r="U195" t="inlineStr">
         <is>
@@ -11022,7 +11022,7 @@
         <v>2</v>
       </c>
       <c r="N196" t="n">
-        <v>2.11</v>
+        <v>2.111</v>
       </c>
       <c r="O196" t="inlineStr">
         <is>
@@ -11188,7 +11188,7 @@
         <v>2</v>
       </c>
       <c r="N199" t="n">
-        <v>3.59</v>
+        <v>3.588</v>
       </c>
       <c r="O199" t="inlineStr">
         <is>
@@ -11202,7 +11202,7 @@
         <v>13</v>
       </c>
       <c r="T199" t="n">
-        <v>2.15</v>
+        <v>2.154</v>
       </c>
       <c r="U199" t="inlineStr">
         <is>
@@ -11245,7 +11245,7 @@
         <v>3</v>
       </c>
       <c r="N200" t="n">
-        <v>2.64</v>
+        <v>2.636</v>
       </c>
       <c r="O200" t="inlineStr">
         <is>
@@ -11407,7 +11407,7 @@
         <v>1</v>
       </c>
       <c r="N205" t="n">
-        <v>2.69</v>
+        <v>2.692</v>
       </c>
       <c r="O205" t="inlineStr">
         <is>
@@ -11421,7 +11421,7 @@
         <v>22</v>
       </c>
       <c r="T205" t="n">
-        <v>1.45</v>
+        <v>1.455</v>
       </c>
       <c r="U205" t="inlineStr">
         <is>
@@ -11479,7 +11479,7 @@
         <v>3</v>
       </c>
       <c r="N206" t="n">
-        <v>2.82</v>
+        <v>2.818</v>
       </c>
       <c r="O206" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
         <v>2</v>
       </c>
       <c r="N208" t="n">
-        <v>2.63</v>
+        <v>2.632</v>
       </c>
       <c r="O208" t="inlineStr">
         <is>
@@ -11610,7 +11610,7 @@
         <v>17</v>
       </c>
       <c r="T208" t="n">
-        <v>1.71</v>
+        <v>1.706</v>
       </c>
       <c r="U208" t="inlineStr">
         <is>
@@ -11804,7 +11804,7 @@
         <v>6</v>
       </c>
       <c r="W211" t="n">
-        <v>1.83</v>
+        <v>1.833</v>
       </c>
       <c r="X211" t="inlineStr">
         <is>
@@ -11877,7 +11877,7 @@
         <v>1</v>
       </c>
       <c r="N213" t="n">
-        <v>3.67</v>
+        <v>3.667</v>
       </c>
       <c r="O213" t="inlineStr">
         <is>
@@ -11927,7 +11927,7 @@
         <v>2</v>
       </c>
       <c r="N214" t="n">
-        <v>2.58</v>
+        <v>2.583</v>
       </c>
       <c r="O214" t="inlineStr">
         <is>
@@ -11941,7 +11941,7 @@
         <v>24</v>
       </c>
       <c r="T214" t="n">
-        <v>1.46</v>
+        <v>1.458</v>
       </c>
       <c r="U214" t="inlineStr">
         <is>
@@ -11952,7 +11952,7 @@
         <v>12</v>
       </c>
       <c r="W214" t="n">
-        <v>2.58</v>
+        <v>2.583</v>
       </c>
       <c r="X214" t="inlineStr">
         <is>
@@ -12005,7 +12005,7 @@
         <v>7</v>
       </c>
       <c r="N215" t="n">
-        <v>1.62</v>
+        <v>1.615</v>
       </c>
       <c r="O215" t="inlineStr">
         <is>
@@ -12019,7 +12019,7 @@
         <v>6</v>
       </c>
       <c r="T215" t="n">
-        <v>1.17</v>
+        <v>1.167</v>
       </c>
       <c r="U215" t="inlineStr">
         <is>
@@ -12030,7 +12030,7 @@
         <v>11</v>
       </c>
       <c r="W215" t="n">
-        <v>2.36</v>
+        <v>2.364</v>
       </c>
       <c r="X215" t="inlineStr">
         <is>
@@ -12147,7 +12147,7 @@
         <v>1</v>
       </c>
       <c r="N217" t="n">
-        <v>2.86</v>
+        <v>2.857</v>
       </c>
       <c r="O217" t="inlineStr">
         <is>
@@ -12161,7 +12161,7 @@
         <v>32</v>
       </c>
       <c r="T217" t="n">
-        <v>1.59</v>
+        <v>1.594</v>
       </c>
       <c r="U217" t="inlineStr">
         <is>
@@ -12172,7 +12172,7 @@
         <v>23</v>
       </c>
       <c r="W217" t="n">
-        <v>2.43</v>
+        <v>2.435</v>
       </c>
       <c r="X217" t="inlineStr">
         <is>
@@ -12216,7 +12216,7 @@
         <v>15</v>
       </c>
       <c r="N218" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="O218" t="inlineStr">
         <is>
@@ -12230,7 +12230,7 @@
         <v>19</v>
       </c>
       <c r="T218" t="n">
-        <v>1.79</v>
+        <v>1.789</v>
       </c>
       <c r="U218" t="inlineStr">
         <is>
@@ -12241,7 +12241,7 @@
         <v>17</v>
       </c>
       <c r="W218" t="n">
-        <v>2.47</v>
+        <v>2.471</v>
       </c>
       <c r="X218" t="inlineStr">
         <is>
@@ -12341,7 +12341,7 @@
         <v>4</v>
       </c>
       <c r="N220" t="n">
-        <v>2.76</v>
+        <v>2.765</v>
       </c>
       <c r="O220" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
         <v>1</v>
       </c>
       <c r="N225" t="n">
-        <v>2.77</v>
+        <v>2.769</v>
       </c>
       <c r="O225" t="inlineStr">
         <is>
@@ -12569,7 +12569,7 @@
         <v>1</v>
       </c>
       <c r="N226" t="n">
-        <v>1.67</v>
+        <v>1.667</v>
       </c>
       <c r="O226" t="inlineStr">
         <is>
@@ -12580,7 +12580,7 @@
         <v>23</v>
       </c>
       <c r="T226" t="n">
-        <v>1.52</v>
+        <v>1.522</v>
       </c>
       <c r="U226" t="inlineStr">
         <is>
@@ -12591,7 +12591,7 @@
         <v>6</v>
       </c>
       <c r="W226" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="X226" t="inlineStr">
         <is>
@@ -12641,7 +12641,7 @@
         <v>1</v>
       </c>
       <c r="N227" t="n">
-        <v>2.64</v>
+        <v>2.643</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -12655,7 +12655,7 @@
         <v>13</v>
       </c>
       <c r="T227" t="n">
-        <v>1.54</v>
+        <v>1.538</v>
       </c>
       <c r="U227" t="inlineStr">
         <is>
@@ -12666,7 +12666,7 @@
         <v>6</v>
       </c>
       <c r="W227" t="n">
-        <v>2.66</v>
+        <v>2.333</v>
       </c>
       <c r="X227" t="inlineStr">
         <is>
@@ -12710,7 +12710,7 @@
         <v>3</v>
       </c>
       <c r="N228" t="n">
-        <v>1.56</v>
+        <v>1.556</v>
       </c>
       <c r="O228" t="inlineStr">
         <is>
@@ -13063,7 +13063,7 @@
         <v>23</v>
       </c>
       <c r="T236" t="n">
-        <v>1.38</v>
+        <v>1.348</v>
       </c>
       <c r="U236" t="inlineStr">
         <is>
@@ -13116,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="N237" t="n">
-        <v>2.58</v>
+        <v>2.583</v>
       </c>
       <c r="O237" t="inlineStr">
         <is>
@@ -13130,7 +13130,7 @@
         <v>31</v>
       </c>
       <c r="T237" t="n">
-        <v>1.74</v>
+        <v>1.742</v>
       </c>
       <c r="U237" t="inlineStr">
         <is>
@@ -13141,7 +13141,7 @@
         <v>8</v>
       </c>
       <c r="W237" t="n">
-        <v>2.38</v>
+        <v>2.375</v>
       </c>
       <c r="X237" t="inlineStr">
         <is>
@@ -13173,7 +13173,7 @@
         <v>3</v>
       </c>
       <c r="N238" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="O238" t="inlineStr">
         <is>
@@ -13248,7 +13248,7 @@
         <v>17</v>
       </c>
       <c r="T239" t="n">
-        <v>1.76</v>
+        <v>1.765</v>
       </c>
       <c r="U239" t="inlineStr">
         <is>
@@ -13312,7 +13312,7 @@
         <v>4</v>
       </c>
       <c r="N240" t="n">
-        <v>2.71</v>
+        <v>2.714</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
@@ -13685,7 +13685,7 @@
         <v>1</v>
       </c>
       <c r="N248" t="n">
-        <v>2.71</v>
+        <v>2.714</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
@@ -13757,7 +13757,7 @@
         <v>19</v>
       </c>
       <c r="T250" t="n">
-        <v>1.53</v>
+        <v>1.526</v>
       </c>
       <c r="U250" t="inlineStr">
         <is>
@@ -13840,7 +13840,7 @@
         <v>6</v>
       </c>
       <c r="W251" t="n">
-        <v>1.83</v>
+        <v>1.833</v>
       </c>
       <c r="X251" t="inlineStr">
         <is>
@@ -13887,7 +13887,7 @@
         <v>2</v>
       </c>
       <c r="N252" t="n">
-        <v>2.67</v>
+        <v>2.667</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -13953,7 +13953,7 @@
         <v>6</v>
       </c>
       <c r="T253" t="n">
-        <v>2.33</v>
+        <v>2.333</v>
       </c>
       <c r="U253" t="inlineStr">
         <is>
@@ -14064,7 +14064,7 @@
         <v>11</v>
       </c>
       <c r="T255" t="n">
-        <v>2.36</v>
+        <v>2.364</v>
       </c>
       <c r="U255" t="inlineStr">
         <is>
@@ -14075,7 +14075,7 @@
         <v>14</v>
       </c>
       <c r="W255" t="n">
-        <v>2.64</v>
+        <v>2.643</v>
       </c>
       <c r="X255" t="inlineStr">
         <is>
@@ -14175,7 +14175,7 @@
         <v>1</v>
       </c>
       <c r="N258" t="n">
-        <v>3.58</v>
+        <v>3.583</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Count each written score as one attempt.
Serve, receive, and freeball ratings divide by how many grades were written, including zeros, instead of the attempt total typed on the sheet.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/volleyball_stats.xlsx
+++ b/volleyball_stats.xlsx
@@ -706,7 +706,7 @@
         <v>0.133</v>
       </c>
       <c r="K3" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="L3" t="n">
         <v>9</v>
@@ -715,7 +715,7 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>3.895</v>
+        <v>3.364</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
         <v>0.4</v>
       </c>
       <c r="K14" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L14" t="n">
         <v>9</v>
@@ -1224,7 +1224,7 @@
         <v>3</v>
       </c>
       <c r="N14" t="n">
-        <v>2.783</v>
+        <v>2.909</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="T16" t="n">
-        <v>1.368</v>
+        <v>1.182</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -1416,10 +1416,10 @@
         </is>
       </c>
       <c r="S17" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T17" t="n">
-        <v>1.769</v>
+        <v>1.917</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -1543,7 +1543,7 @@
         <v>0.263</v>
       </c>
       <c r="K19" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L19" t="n">
         <v>8</v>
@@ -1552,7 +1552,7 @@
         <v>5</v>
       </c>
       <c r="N19" t="n">
-        <v>2.667</v>
+        <v>2.824</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1809,7 +1809,7 @@
         <v>2</v>
       </c>
       <c r="K26" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L26" t="n">
         <v>2</v>
@@ -1818,7 +1818,7 @@
         <v>4</v>
       </c>
       <c r="N26" t="n">
-        <v>2</v>
+        <v>1.714</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -1934,7 +1934,7 @@
         <v>-0.143</v>
       </c>
       <c r="K28" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L28" t="n">
         <v>6</v>
@@ -1943,7 +1943,7 @@
         <v>1</v>
       </c>
       <c r="N28" t="n">
-        <v>3.056</v>
+        <v>3.235</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2509,10 +2509,10 @@
         </is>
       </c>
       <c r="S39" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T39" t="n">
-        <v>1.455</v>
+        <v>1.333</v>
       </c>
       <c r="U39" t="inlineStr">
         <is>
@@ -4005,7 +4005,7 @@
         <v>0.222</v>
       </c>
       <c r="K67" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L67" t="n">
         <v>3</v>
@@ -4014,7 +4014,7 @@
         <v>3</v>
       </c>
       <c r="N67" t="n">
-        <v>2.385</v>
+        <v>2.583</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -4025,10 +4025,10 @@
         <v>2</v>
       </c>
       <c r="S67" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="T67" t="n">
-        <v>1.75</v>
+        <v>1.944</v>
       </c>
       <c r="U67" t="inlineStr">
         <is>
@@ -4612,7 +4612,7 @@
         <v>-0.5</v>
       </c>
       <c r="K79" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L79" t="n">
         <v>2</v>
@@ -4621,7 +4621,7 @@
         <v>2</v>
       </c>
       <c r="N79" t="n">
-        <v>3.375</v>
+        <v>3</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -4698,10 +4698,10 @@
         <v>1</v>
       </c>
       <c r="S80" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T80" t="n">
-        <v>0.5</v>
+        <v>0.667</v>
       </c>
       <c r="U80" t="inlineStr">
         <is>
@@ -5459,10 +5459,10 @@
         </is>
       </c>
       <c r="S97" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="T97" t="n">
-        <v>1.3</v>
+        <v>1.368</v>
       </c>
       <c r="U97" t="inlineStr">
         <is>
@@ -5742,7 +5742,7 @@
         <v>-0.05</v>
       </c>
       <c r="K101" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L101" t="n">
         <v>6</v>
@@ -5751,7 +5751,7 @@
         <v>7</v>
       </c>
       <c r="N101" t="n">
-        <v>2.429</v>
+        <v>2.55</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
@@ -6888,7 +6888,7 @@
         <v>-0.5</v>
       </c>
       <c r="K119" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L119" t="n">
         <v>1</v>
@@ -6897,7 +6897,7 @@
         <v>1</v>
       </c>
       <c r="N119" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
         <v>1</v>
       </c>
       <c r="K133" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L133" t="n">
         <v>1</v>
@@ -7632,7 +7632,7 @@
         <v>3</v>
       </c>
       <c r="N133" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -9142,13 +9142,13 @@
         <v>0</v>
       </c>
       <c r="K161" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L161" t="n">
         <v>6</v>
       </c>
       <c r="N161" t="n">
-        <v>3.12</v>
+        <v>3</v>
       </c>
       <c r="O161" t="inlineStr">
         <is>
@@ -10566,13 +10566,13 @@
         <v>10</v>
       </c>
       <c r="K188" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M188" t="n">
         <v>1</v>
       </c>
       <c r="N188" t="n">
-        <v>2.25</v>
+        <v>1.8</v>
       </c>
       <c r="O188" t="inlineStr">
         <is>
@@ -11429,10 +11429,10 @@
         </is>
       </c>
       <c r="V205" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W205" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="X205" t="inlineStr">
         <is>
@@ -13060,10 +13060,10 @@
         </is>
       </c>
       <c r="S236" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="T236" t="n">
-        <v>1.348</v>
+        <v>1.292</v>
       </c>
       <c r="U236" t="inlineStr">
         <is>

</xml_diff>